<commit_message>
Apr 22 2026 update
</commit_message>
<xml_diff>
--- a/static/data/source/state_and_local_public_education_employment.xlsx
+++ b/static/data/source/state_and_local_public_education_employment.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="L:\TPC\Scratch\Garriga\D drive transfer\SEM BLS Update\Tables\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM BLS Update\Tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56FD35CE-2CF3-4E34-B5D6-DC37C524233D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18128782-8682-4916-8D65-EF4258F4BD3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2685" yWindow="2685" windowWidth="16200" windowHeight="9270" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TABLE_1" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="223">
   <si>
     <t>Geography</t>
   </si>
@@ -533,6 +533,9 @@
     <t>01/01/2026</t>
   </si>
   <si>
+    <t>02/01/2026</t>
+  </si>
+  <si>
     <t>United States</t>
   </si>
   <si>
@@ -1020,10 +1023,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A4:FN56"/>
+  <dimension ref="A4:FO56"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="4" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -1534,10 +1537,13 @@
       <c r="FN4" t="s">
         <v>169</v>
       </c>
+      <c r="FO4" t="s">
+        <v>170</v>
+      </c>
     </row>
-    <row r="5" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B5">
         <v>10186.6</v>
@@ -2046,10 +2052,13 @@
       <c r="FN5">
         <v>10913.3</v>
       </c>
+      <c r="FO5">
+        <v>11238.1</v>
+      </c>
     </row>
-    <row r="6" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B6">
         <v>162</v>
@@ -2556,12 +2565,15 @@
         <v>184.2</v>
       </c>
       <c r="FN6">
-        <v>180.9</v>
+        <v>182.8</v>
+      </c>
+      <c r="FO6">
+        <v>185.4</v>
       </c>
     </row>
-    <row r="7" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B7">
         <v>30.4</v>
@@ -3070,10 +3082,13 @@
       <c r="FN7">
         <v>27.1</v>
       </c>
+      <c r="FO7">
+        <v>27.9</v>
+      </c>
     </row>
-    <row r="8" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B8">
         <v>190.5</v>
@@ -3582,10 +3597,13 @@
       <c r="FN8">
         <v>191.6</v>
       </c>
+      <c r="FO8">
+        <v>200.7</v>
+      </c>
     </row>
-    <row r="9" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B9">
         <v>102.9</v>
@@ -4094,10 +4112,13 @@
       <c r="FN9">
         <v>95.3</v>
       </c>
+      <c r="FO9">
+        <v>96.9</v>
+      </c>
     </row>
-    <row r="10" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B10">
         <v>1132.3</v>
@@ -4604,12 +4625,15 @@
         <v>1274</v>
       </c>
       <c r="FN10">
-        <v>1254.5</v>
+        <v>1254.7</v>
+      </c>
+      <c r="FO10">
+        <v>1267.8</v>
       </c>
     </row>
-    <row r="11" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B11">
         <v>184.5</v>
@@ -5118,10 +5142,13 @@
       <c r="FN11">
         <v>236.7</v>
       </c>
+      <c r="FO11">
+        <v>245.7</v>
+      </c>
     </row>
-    <row r="12" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B12">
         <v>122.1</v>
@@ -5630,10 +5657,13 @@
       <c r="FN12">
         <v>124.8</v>
       </c>
+      <c r="FO12">
+        <v>125.7</v>
+      </c>
     </row>
-    <row r="13" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B13">
         <v>30.2</v>
@@ -6140,20 +6170,20 @@
         <v>39.700000000000003</v>
       </c>
       <c r="FN13">
-        <v>37.5</v>
+        <v>38</v>
+      </c>
+      <c r="FO13">
+        <v>39.5</v>
       </c>
     </row>
-    <row r="14" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>179</v>
-      </c>
-      <c r="FK14">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
-    <row r="15" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B15">
         <v>490.3</v>
@@ -6660,12 +6690,15 @@
         <v>494.6</v>
       </c>
       <c r="FN15">
-        <v>491.1</v>
+        <v>491.7</v>
+      </c>
+      <c r="FO15">
+        <v>501</v>
       </c>
     </row>
-    <row r="16" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B16">
         <v>345.9</v>
@@ -7174,18 +7207,18 @@
       <c r="FN16">
         <v>351</v>
       </c>
+      <c r="FO16">
+        <v>353.8</v>
+      </c>
     </row>
-    <row r="17" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>182</v>
-      </c>
-      <c r="FK17">
-        <v>0</v>
+        <v>183</v>
       </c>
     </row>
-    <row r="18" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B18">
         <v>52.4</v>
@@ -7694,10 +7727,13 @@
       <c r="FN18">
         <v>62.1</v>
       </c>
+      <c r="FO18">
+        <v>64.099999999999994</v>
+      </c>
     </row>
-    <row r="19" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B19">
         <v>435.1</v>
@@ -8204,12 +8240,15 @@
         <v>470.8</v>
       </c>
       <c r="FN19">
-        <v>456.1</v>
+        <v>448</v>
+      </c>
+      <c r="FO19">
+        <v>470.7</v>
       </c>
     </row>
-    <row r="20" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B20">
         <v>236</v>
@@ -8716,12 +8755,15 @@
         <v>226.5</v>
       </c>
       <c r="FN20">
-        <v>220.1</v>
+        <v>219.7</v>
+      </c>
+      <c r="FO20">
+        <v>228</v>
       </c>
     </row>
-    <row r="21" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B21">
         <v>139</v>
@@ -9230,10 +9272,13 @@
       <c r="FN21">
         <v>147.9</v>
       </c>
+      <c r="FO21">
+        <v>150.5</v>
+      </c>
     </row>
-    <row r="22" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B22">
         <v>135.1</v>
@@ -9742,10 +9787,13 @@
       <c r="FN22">
         <v>136.9</v>
       </c>
+      <c r="FO22">
+        <v>140.19999999999999</v>
+      </c>
     </row>
-    <row r="23" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B23">
         <v>171.5</v>
@@ -10254,10 +10302,13 @@
       <c r="FN23">
         <v>160.4</v>
       </c>
+      <c r="FO23">
+        <v>163.9</v>
+      </c>
     </row>
-    <row r="24" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B24">
         <v>160.9</v>
@@ -10766,10 +10817,13 @@
       <c r="FN24">
         <v>150.5</v>
       </c>
+      <c r="FO24">
+        <v>152.6</v>
+      </c>
     </row>
-    <row r="25" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B25">
         <v>50.7</v>
@@ -11276,12 +11330,15 @@
         <v>49.5</v>
       </c>
       <c r="FN25">
-        <v>47.9</v>
+        <v>47.8</v>
+      </c>
+      <c r="FO25">
+        <v>49.1</v>
       </c>
     </row>
-    <row r="26" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B26">
         <v>194.8</v>
@@ -11790,10 +11847,13 @@
       <c r="FN26">
         <v>213.8</v>
       </c>
+      <c r="FO26">
+        <v>227.8</v>
+      </c>
     </row>
-    <row r="27" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B27">
         <v>216.5</v>
@@ -12302,10 +12362,13 @@
       <c r="FN27">
         <v>241.8</v>
       </c>
+      <c r="FO27">
+        <v>249.2</v>
+      </c>
     </row>
-    <row r="28" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B28">
         <v>326.8</v>
@@ -12814,10 +12877,13 @@
       <c r="FN28">
         <v>317.8</v>
       </c>
+      <c r="FO28">
+        <v>333.7</v>
+      </c>
     </row>
-    <row r="29" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B29">
         <v>201</v>
@@ -13326,10 +13392,13 @@
       <c r="FN29">
         <v>213.6</v>
       </c>
+      <c r="FO29">
+        <v>217.2</v>
+      </c>
     </row>
-    <row r="30" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B30">
         <v>106.5</v>
@@ -13838,15 +13907,18 @@
       <c r="FN30">
         <v>101.9</v>
       </c>
+      <c r="FO30">
+        <v>104.4</v>
+      </c>
     </row>
-    <row r="31" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
-    <row r="32" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B32">
         <v>42.2</v>
@@ -14344,7 +14416,7 @@
         <v>41.3</v>
       </c>
       <c r="FK32">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="FL32">
         <v>42.5</v>
@@ -14355,10 +14427,13 @@
       <c r="FN32">
         <v>41.6</v>
       </c>
+      <c r="FO32">
+        <v>42.6</v>
+      </c>
     </row>
-    <row r="33" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B33">
         <v>86.4</v>
@@ -14856,7 +14931,7 @@
         <v>94.8</v>
       </c>
       <c r="FK33">
-        <v>98.4</v>
+        <v>0</v>
       </c>
       <c r="FL33">
         <v>98.9</v>
@@ -14867,10 +14942,13 @@
       <c r="FN33">
         <v>94.7</v>
       </c>
+      <c r="FO33">
+        <v>97.5</v>
+      </c>
     </row>
-    <row r="34" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B34">
         <v>66.2</v>
@@ -15368,7 +15446,7 @@
         <v>88.5</v>
       </c>
       <c r="FK34">
-        <v>89.1</v>
+        <v>0</v>
       </c>
       <c r="FL34">
         <v>90.4</v>
@@ -15379,10 +15457,13 @@
       <c r="FN34">
         <v>81.400000000000006</v>
       </c>
+      <c r="FO34">
+        <v>89.8</v>
+      </c>
     </row>
-    <row r="35" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B35">
         <v>47.3</v>
@@ -15880,7 +15961,7 @@
         <v>42.7</v>
       </c>
       <c r="FK35">
-        <v>43.8</v>
+        <v>0</v>
       </c>
       <c r="FL35">
         <v>44.1</v>
@@ -15891,10 +15972,13 @@
       <c r="FN35">
         <v>41.5</v>
       </c>
+      <c r="FO35">
+        <v>43.9</v>
+      </c>
     </row>
-    <row r="36" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B36">
         <v>314.2</v>
@@ -16392,7 +16476,7 @@
         <v>315.10000000000002</v>
       </c>
       <c r="FK36">
-        <v>336.1</v>
+        <v>0</v>
       </c>
       <c r="FL36">
         <v>339.4</v>
@@ -16401,12 +16485,15 @@
         <v>338</v>
       </c>
       <c r="FN36">
-        <v>325.7</v>
+        <v>325.8</v>
+      </c>
+      <c r="FO36">
+        <v>337.7</v>
       </c>
     </row>
-    <row r="37" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B37">
         <v>77.3</v>
@@ -16856,13 +16943,13 @@
         <v>80.2</v>
       </c>
       <c r="EU37">
-        <v>72.900000000000006</v>
+        <v>71.5</v>
       </c>
       <c r="EV37">
-        <v>49.9</v>
+        <v>63.2</v>
       </c>
       <c r="EW37">
-        <v>72.099999999999994</v>
+        <v>71.400000000000006</v>
       </c>
       <c r="EX37">
         <v>78.5</v>
@@ -16904,7 +16991,7 @@
         <v>77.599999999999994</v>
       </c>
       <c r="FK37">
-        <v>78.7</v>
+        <v>0</v>
       </c>
       <c r="FL37">
         <v>80</v>
@@ -16915,10 +17002,13 @@
       <c r="FN37">
         <v>77.599999999999994</v>
       </c>
+      <c r="FO37">
+        <v>80.099999999999994</v>
+      </c>
     </row>
-    <row r="38" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B38">
         <v>634.6</v>
@@ -17416,7 +17506,7 @@
         <v>666.1</v>
       </c>
       <c r="FK38">
-        <v>694.1</v>
+        <v>0</v>
       </c>
       <c r="FL38">
         <v>700.2</v>
@@ -17425,12 +17515,15 @@
         <v>700.7</v>
       </c>
       <c r="FN38">
-        <v>686.9</v>
+        <v>683.2</v>
+      </c>
+      <c r="FO38">
+        <v>700.7</v>
       </c>
     </row>
-    <row r="39" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B39">
         <v>340.2</v>
@@ -17928,7 +18021,7 @@
         <v>337.1</v>
       </c>
       <c r="FK39">
-        <v>341.2</v>
+        <v>0</v>
       </c>
       <c r="FL39">
         <v>345.2</v>
@@ -17939,10 +18032,13 @@
       <c r="FN39">
         <v>336.3</v>
       </c>
+      <c r="FO39">
+        <v>343.4</v>
+      </c>
     </row>
-    <row r="40" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B40">
         <v>37.1</v>
@@ -18440,7 +18536,7 @@
         <v>38.799999999999997</v>
       </c>
       <c r="FK40">
-        <v>40.200000000000003</v>
+        <v>0</v>
       </c>
       <c r="FL40">
         <v>40.700000000000003</v>
@@ -18451,10 +18547,13 @@
       <c r="FN40">
         <v>40</v>
       </c>
+      <c r="FO40">
+        <v>41.1</v>
+      </c>
     </row>
-    <row r="41" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B41">
         <v>374.9</v>
@@ -18952,7 +19051,7 @@
         <v>383.8</v>
       </c>
       <c r="FK41">
-        <v>399.7</v>
+        <v>0</v>
       </c>
       <c r="FL41">
         <v>402.9</v>
@@ -18961,12 +19060,15 @@
         <v>397.1</v>
       </c>
       <c r="FN41">
-        <v>388.7</v>
+        <v>387.6</v>
+      </c>
+      <c r="FO41">
+        <v>395.8</v>
       </c>
     </row>
-    <row r="42" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B42">
         <v>146.69999999999999</v>
@@ -19464,7 +19566,7 @@
         <v>154.1</v>
       </c>
       <c r="FK42">
-        <v>158</v>
+        <v>0</v>
       </c>
       <c r="FL42">
         <v>159</v>
@@ -19475,10 +19577,13 @@
       <c r="FN42">
         <v>148.9</v>
       </c>
+      <c r="FO42">
+        <v>157.19999999999999</v>
+      </c>
     </row>
-    <row r="43" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B43">
         <v>130.30000000000001</v>
@@ -19976,7 +20081,7 @@
         <v>127.9</v>
       </c>
       <c r="FK43">
-        <v>138.6</v>
+        <v>0</v>
       </c>
       <c r="FL43">
         <v>139.69999999999999</v>
@@ -19987,10 +20092,13 @@
       <c r="FN43">
         <v>137</v>
       </c>
+      <c r="FO43">
+        <v>139.30000000000001</v>
+      </c>
     </row>
-    <row r="44" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B44">
         <v>343.9</v>
@@ -20488,7 +20596,7 @@
         <v>332.1</v>
       </c>
       <c r="FK44">
-        <v>340.5</v>
+        <v>0</v>
       </c>
       <c r="FL44">
         <v>344.2</v>
@@ -20499,10 +20607,13 @@
       <c r="FN44">
         <v>327.5</v>
       </c>
+      <c r="FO44">
+        <v>338.3</v>
+      </c>
     </row>
-    <row r="45" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B45">
         <v>31.3</v>
@@ -21000,7 +21111,7 @@
         <v>29</v>
       </c>
       <c r="FK45">
-        <v>29.4</v>
+        <v>0</v>
       </c>
       <c r="FL45">
         <v>30.1</v>
@@ -21011,10 +21122,13 @@
       <c r="FN45">
         <v>29.1</v>
       </c>
+      <c r="FO45">
+        <v>30.2</v>
+      </c>
     </row>
-    <row r="46" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B46">
         <v>159.1</v>
@@ -21512,7 +21626,7 @@
         <v>176.5</v>
       </c>
       <c r="FK46">
-        <v>177.7</v>
+        <v>0</v>
       </c>
       <c r="FL46">
         <v>178.8</v>
@@ -21523,10 +21637,13 @@
       <c r="FN46">
         <v>174.4</v>
       </c>
+      <c r="FO46">
+        <v>177.9</v>
+      </c>
     </row>
-    <row r="47" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B47">
         <v>35</v>
@@ -22024,7 +22141,7 @@
         <v>37.799999999999997</v>
       </c>
       <c r="FK47">
-        <v>38.9</v>
+        <v>0</v>
       </c>
       <c r="FL47">
         <v>39.1</v>
@@ -22035,10 +22152,13 @@
       <c r="FN47">
         <v>37.299999999999997</v>
       </c>
+      <c r="FO47">
+        <v>38.799999999999997</v>
+      </c>
     </row>
-    <row r="48" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B48">
         <v>194.7</v>
@@ -22536,7 +22656,7 @@
         <v>214.9</v>
       </c>
       <c r="FK48">
-        <v>220.5</v>
+        <v>0</v>
       </c>
       <c r="FL48">
         <v>222.2</v>
@@ -22547,10 +22667,13 @@
       <c r="FN48">
         <v>208.3</v>
       </c>
+      <c r="FO48">
+        <v>220.4</v>
+      </c>
     </row>
-    <row r="49" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B49">
         <v>1028</v>
@@ -23048,7 +23171,7 @@
         <v>1182.9000000000001</v>
       </c>
       <c r="FK49">
-        <v>1219.4000000000001</v>
+        <v>0</v>
       </c>
       <c r="FL49">
         <v>1227</v>
@@ -23057,12 +23180,15 @@
         <v>1223.5999999999999</v>
       </c>
       <c r="FN49">
-        <v>1192.0999999999999</v>
+        <v>1190.2</v>
+      </c>
+      <c r="FO49">
+        <v>1218.3</v>
       </c>
     </row>
-    <row r="50" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B50">
         <v>109.5</v>
@@ -23560,7 +23686,7 @@
         <v>132.6</v>
       </c>
       <c r="FK50">
-        <v>135.80000000000001</v>
+        <v>0</v>
       </c>
       <c r="FL50">
         <v>136.80000000000001</v>
@@ -23571,10 +23697,13 @@
       <c r="FN50">
         <v>133.5</v>
       </c>
+      <c r="FO50">
+        <v>136.5</v>
+      </c>
     </row>
-    <row r="51" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B51">
         <v>33</v>
@@ -24072,7 +24201,7 @@
         <v>31.4</v>
       </c>
       <c r="FK51">
-        <v>32.700000000000003</v>
+        <v>0</v>
       </c>
       <c r="FL51">
         <v>33.1</v>
@@ -24081,12 +24210,15 @@
         <v>32.4</v>
       </c>
       <c r="FN51">
-        <v>31.4</v>
+        <v>31.2</v>
+      </c>
+      <c r="FO51">
+        <v>33</v>
       </c>
     </row>
-    <row r="52" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B52">
         <v>311.5</v>
@@ -24584,7 +24716,7 @@
         <v>336.8</v>
       </c>
       <c r="FK52">
-        <v>347.7</v>
+        <v>0</v>
       </c>
       <c r="FL52">
         <v>353.5</v>
@@ -24593,12 +24725,15 @@
         <v>348.2</v>
       </c>
       <c r="FN52">
-        <v>334.5</v>
+        <v>334.6</v>
+      </c>
+      <c r="FO52">
+        <v>351.9</v>
       </c>
     </row>
-    <row r="53" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B53">
         <v>240.6</v>
@@ -25096,7 +25231,7 @@
         <v>247.3</v>
       </c>
       <c r="FK53">
-        <v>261.5</v>
+        <v>0</v>
       </c>
       <c r="FL53">
         <v>266.5</v>
@@ -25107,10 +25242,13 @@
       <c r="FN53">
         <v>264.89999999999998</v>
       </c>
+      <c r="FO53">
+        <v>267.39999999999998</v>
+      </c>
     </row>
-    <row r="54" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B54">
         <v>68.900000000000006</v>
@@ -25608,7 +25746,7 @@
         <v>60.6</v>
       </c>
       <c r="FK54">
-        <v>62.8</v>
+        <v>0</v>
       </c>
       <c r="FL54">
         <v>63.6</v>
@@ -25619,10 +25757,13 @@
       <c r="FN54">
         <v>58.6</v>
       </c>
+      <c r="FO54">
+        <v>61.8</v>
+      </c>
     </row>
-    <row r="55" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B55">
         <v>199.2</v>
@@ -26120,7 +26261,7 @@
         <v>204.3</v>
       </c>
       <c r="FK55">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="FL55">
         <v>213.2</v>
@@ -26129,12 +26270,15 @@
         <v>211.6</v>
       </c>
       <c r="FN55">
-        <v>200.2</v>
+        <v>200.1</v>
+      </c>
+      <c r="FO55">
+        <v>210.8</v>
       </c>
     </row>
-    <row r="56" spans="1:170" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:171" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B56">
         <v>31.4</v>
@@ -26632,7 +26776,7 @@
         <v>30</v>
       </c>
       <c r="FK56">
-        <v>31.2</v>
+        <v>0</v>
       </c>
       <c r="FL56">
         <v>31.2</v>
@@ -26642,6 +26786,9 @@
       </c>
       <c r="FN56">
         <v>29</v>
+      </c>
+      <c r="FO56">
+        <v>31.3</v>
       </c>
     </row>
   </sheetData>
@@ -26652,10 +26799,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A4:FB56"/>
+  <dimension ref="A4:FC56"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="4" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -27130,10 +27277,13 @@
       <c r="FB4" t="s">
         <v>169</v>
       </c>
+      <c r="FC4" t="s">
+        <v>170</v>
+      </c>
     </row>
-    <row r="5" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B5">
         <v>-0.32100995425363399</v>
@@ -27606,10 +27756,13 @@
       <c r="FB5">
         <v>1.92462790527031E-2</v>
       </c>
+      <c r="FC5">
+        <v>-1.3345670664436499E-2</v>
+      </c>
     </row>
-    <row r="6" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B6">
         <v>-0.37037037037036702</v>
@@ -28080,12 +28233,15 @@
         <v>1.7117614577581399</v>
       </c>
       <c r="FB6">
-        <v>1.7435320584926699</v>
+        <v>2.8121484814398201</v>
+      </c>
+      <c r="FC6">
+        <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B7">
         <v>-0.32894736842105698</v>
@@ -28558,10 +28714,13 @@
       <c r="FB7">
         <v>-2.5179856115107899</v>
       </c>
+      <c r="FC7">
+        <v>-3.125</v>
+      </c>
     </row>
-    <row r="8" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B8">
         <v>1.67979002624671</v>
@@ -29034,10 +29193,13 @@
       <c r="FB8">
         <v>-4.0080160320641296</v>
       </c>
+      <c r="FC8">
+        <v>-2.4781341107871802</v>
+      </c>
     </row>
-    <row r="9" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B9">
         <v>0.194363459669571</v>
@@ -29510,10 +29672,13 @@
       <c r="FB9">
         <v>-0.31380753138075002</v>
       </c>
+      <c r="FC9">
+        <v>-0.30864197530863902</v>
+      </c>
     </row>
-    <row r="10" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B10">
         <v>-0.55638964938620095</v>
@@ -29984,12 +30149,15 @@
         <v>-2.2781314719644099</v>
       </c>
       <c r="FB10">
-        <v>-3.3661993529502299</v>
+        <v>-3.3507934062547999</v>
+      </c>
+      <c r="FC10">
+        <v>-1.8350754936120801</v>
       </c>
     </row>
-    <row r="11" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B11">
         <v>0.43360433604336701</v>
@@ -30462,10 +30630,13 @@
       <c r="FB11">
         <v>1.67525773195877</v>
       </c>
+      <c r="FC11">
+        <v>1.6970198675496699</v>
+      </c>
     </row>
-    <row r="12" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B12">
         <v>1.06470106470107</v>
@@ -30938,10 +31109,13 @@
       <c r="FB12">
         <v>-0.47846889952153798</v>
       </c>
+      <c r="FC12">
+        <v>-0.238095238095236</v>
+      </c>
     </row>
-    <row r="13" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B13">
         <v>-1.98675496688743</v>
@@ -31412,20 +31586,23 @@
         <v>-0.74999999999999301</v>
       </c>
       <c r="FB13">
-        <v>-1.31578947368421</v>
+        <v>0</v>
+      </c>
+      <c r="FC13">
+        <v>1.54241645244216</v>
       </c>
     </row>
-    <row r="14" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="EY14">
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B15">
         <v>0.877014073016534</v>
@@ -31896,12 +32073,15 @@
         <v>-1.0404161664666001</v>
       </c>
       <c r="FB15">
-        <v>-1.4646869983948501</v>
+        <v>-1.34430176565008</v>
+      </c>
+      <c r="FC15">
+        <v>-0.98814229249011898</v>
       </c>
     </row>
-    <row r="16" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B16">
         <v>-1.3587742122000399</v>
@@ -32374,18 +32554,21 @@
       <c r="FB16">
         <v>0.171232876712335</v>
       </c>
+      <c r="FC16">
+        <v>0.42577348850413199</v>
+      </c>
     </row>
-    <row r="17" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="EY17">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B18">
         <v>3.4351145038167901</v>
@@ -32858,10 +33041,13 @@
       <c r="FB18">
         <v>-1.4285714285714399</v>
       </c>
+      <c r="FC18">
+        <v>-0.927357032457509</v>
+      </c>
     </row>
-    <row r="19" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B19">
         <v>1.33302689037002</v>
@@ -33332,12 +33518,15 @@
         <v>1.3126748439853599</v>
       </c>
       <c r="FB19">
-        <v>1.22059476253884</v>
+        <v>-0.57700843320018302</v>
+      </c>
+      <c r="FC19">
+        <v>1.00858369098712</v>
       </c>
     </row>
-    <row r="20" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B20">
         <v>-1.4830508474576301</v>
@@ -33808,12 +33997,15 @@
         <v>-5.5462885738115002</v>
       </c>
       <c r="FB20">
-        <v>-5.3333333333333197</v>
+        <v>-5.5053763440860299</v>
+      </c>
+      <c r="FC20">
+        <v>-1.6817593790426799</v>
       </c>
     </row>
-    <row r="21" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B21">
         <v>0.14388489208632299</v>
@@ -34286,10 +34478,13 @@
       <c r="FB21">
         <v>0.13540961408261101</v>
       </c>
+      <c r="FC21">
+        <v>-0.26507620941020898</v>
+      </c>
     </row>
-    <row r="22" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B22">
         <v>-0.88823094004440295</v>
@@ -34762,10 +34957,13 @@
       <c r="FB22">
         <v>4.4241037376048897</v>
       </c>
+      <c r="FC22">
+        <v>0.93592512598992905</v>
+      </c>
     </row>
-    <row r="23" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B23">
         <v>-0.34985422740526101</v>
@@ -35238,10 +35436,13 @@
       <c r="FB23">
         <v>0.50125313283206996</v>
       </c>
+      <c r="FC23">
+        <v>-1.1459589867310001</v>
+      </c>
     </row>
-    <row r="24" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B24">
         <v>-3.6047234307023102</v>
@@ -35714,10 +35915,13 @@
       <c r="FB24">
         <v>-6.6401062417013795E-2</v>
       </c>
+      <c r="FC24">
+        <v>-6.54878847413191E-2</v>
+      </c>
     </row>
-    <row r="25" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B25">
         <v>0.98619329388561605</v>
@@ -36188,12 +36392,15 @@
         <v>-1.19760479041916</v>
       </c>
       <c r="FB25">
-        <v>-1.8442622950819501</v>
+        <v>-2.0491803278688399</v>
+      </c>
+      <c r="FC25">
+        <v>-0.80808080808081995</v>
       </c>
     </row>
-    <row r="26" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B26">
         <v>1.4373716632443601</v>
@@ -36666,10 +36873,13 @@
       <c r="FB26">
         <v>0.42273367778301302</v>
       </c>
+      <c r="FC26">
+        <v>0.57395143487858002</v>
+      </c>
     </row>
-    <row r="27" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B27">
         <v>1.10854503464202</v>
@@ -37142,10 +37352,13 @@
       <c r="FB27">
         <v>0.29033596018250402</v>
       </c>
+      <c r="FC27">
+        <v>0.16077170418005499</v>
+      </c>
     </row>
-    <row r="28" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B28">
         <v>-2.4785801713586202</v>
@@ -37618,10 +37831,13 @@
       <c r="FB28">
         <v>2.3840206185567099</v>
       </c>
+      <c r="FC28">
+        <v>2.6769230769230701</v>
+      </c>
     </row>
-    <row r="29" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B29">
         <v>1.1940298507462599</v>
@@ -38094,10 +38310,13 @@
       <c r="FB29">
         <v>1.32827324478179</v>
       </c>
+      <c r="FC29">
+        <v>0.41608876560331798</v>
+      </c>
     </row>
-    <row r="30" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B30">
         <v>0.28169014084506799</v>
@@ -38570,15 +38789,21 @@
       <c r="FB30">
         <v>0.79129574678537196</v>
       </c>
+      <c r="FC30">
+        <v>1.36119298038333E-14</v>
+      </c>
     </row>
-    <row r="31" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>196</v>
+        <v>197</v>
+      </c>
+      <c r="EY31">
+        <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B32">
         <v>3.3175355450236799</v>
@@ -39040,7 +39265,7 @@
         <v>-1.19617224880383</v>
       </c>
       <c r="EY32">
-        <v>-1.1764705882352899</v>
+        <v>0</v>
       </c>
       <c r="EZ32">
         <v>-1.16279069767442</v>
@@ -39051,10 +39276,13 @@
       <c r="FB32">
         <v>-1.18764845605701</v>
       </c>
+      <c r="FC32">
+        <v>-1.16009280742458</v>
+      </c>
     </row>
-    <row r="33" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B33">
         <v>0.69444444444443798</v>
@@ -39516,7 +39744,7 @@
         <v>0.95846645367411198</v>
       </c>
       <c r="EY33">
-        <v>0.40816326530612801</v>
+        <v>0</v>
       </c>
       <c r="EZ33">
         <v>0.712830957230145</v>
@@ -39527,10 +39755,13 @@
       <c r="FB33">
         <v>1.0672358591248701</v>
       </c>
+      <c r="FC33">
+        <v>0.82730093071354405</v>
+      </c>
     </row>
-    <row r="34" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B34">
         <v>2.7190332326283899</v>
@@ -39992,7 +40223,7 @@
         <v>1.02739726027398</v>
       </c>
       <c r="EY34">
-        <v>0.33783783783781901</v>
+        <v>0</v>
       </c>
       <c r="EZ34">
         <v>1.11856823266219</v>
@@ -40003,10 +40234,13 @@
       <c r="FB34">
         <v>1.3698630136986401</v>
       </c>
+      <c r="FC34">
+        <v>0.78563411896745505</v>
+      </c>
     </row>
-    <row r="35" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B35">
         <v>0.21141649048626099</v>
@@ -40468,7 +40702,7 @@
         <v>-2.9545454545454501</v>
       </c>
       <c r="EY35">
-        <v>-3.5242290748898699</v>
+        <v>0</v>
       </c>
       <c r="EZ35">
         <v>-3.7117903930131102</v>
@@ -40479,10 +40713,13 @@
       <c r="FB35">
         <v>-3.4883720930232598</v>
       </c>
+      <c r="FC35">
+        <v>-3.3039647577092501</v>
+      </c>
     </row>
-    <row r="36" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B36">
         <v>2.8007638446849201</v>
@@ -40944,7 +41181,7 @@
         <v>0.286441756842786</v>
       </c>
       <c r="EY36">
-        <v>0.77961019490255601</v>
+        <v>0</v>
       </c>
       <c r="EZ36">
         <v>0.62259116513488499</v>
@@ -40953,12 +41190,15 @@
         <v>0.41592394533570298</v>
       </c>
       <c r="FB36">
-        <v>0.92965602726992802</v>
+        <v>0.96064456151224797</v>
+      </c>
+      <c r="FC36">
+        <v>0.26722090261282</v>
       </c>
     </row>
-    <row r="37" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B37">
         <v>2.8460543337645601</v>
@@ -41372,13 +41612,13 @@
         <v>3.2175032175032001</v>
       </c>
       <c r="EI37">
-        <v>4.4412607449856898</v>
+        <v>2.4355300859598898</v>
       </c>
       <c r="EJ37">
-        <v>-22.03125</v>
+        <v>-1.25</v>
       </c>
       <c r="EK37">
-        <v>1.69252468265161</v>
+        <v>0.70521861777150896</v>
       </c>
       <c r="EL37">
         <v>1.42118863049095</v>
@@ -41408,19 +41648,19 @@
         <v>0.87281795511224103</v>
       </c>
       <c r="EU37">
-        <v>-1.50891632373115</v>
+        <v>0.41958041958041598</v>
       </c>
       <c r="EV37">
-        <v>25.050100200400799</v>
+        <v>-1.26582278481013</v>
       </c>
       <c r="EW37">
-        <v>-1.94174757281552</v>
+        <v>-0.98039215686274905</v>
       </c>
       <c r="EX37">
         <v>-1.1464968152866299</v>
       </c>
       <c r="EY37">
-        <v>-1.625</v>
+        <v>0</v>
       </c>
       <c r="EZ37">
         <v>-1.35635018495684</v>
@@ -41431,10 +41671,13 @@
       <c r="FB37">
         <v>-0.89399744572158701</v>
       </c>
+      <c r="FC37">
+        <v>-1.71779141104295</v>
+      </c>
     </row>
-    <row r="38" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B38">
         <v>-1.4182161991805899</v>
@@ -41896,7 +42139,7 @@
         <v>2.6664611590629002</v>
       </c>
       <c r="EY38">
-        <v>2.6319680615111398</v>
+        <v>0</v>
       </c>
       <c r="EZ38">
         <v>2.6686217008797701</v>
@@ -41905,12 +42148,15 @@
         <v>2.6817116060961399</v>
       </c>
       <c r="FB38">
-        <v>3.5735826296742998</v>
+        <v>3.0156815440289302</v>
+      </c>
+      <c r="FC38">
+        <v>2.0238788584740801</v>
       </c>
     </row>
-    <row r="39" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B39">
         <v>0.20576131687242499</v>
@@ -42372,7 +42618,7 @@
         <v>8.9073634204278898E-2</v>
       </c>
       <c r="EY39">
-        <v>0.205580029368572</v>
+        <v>0</v>
       </c>
       <c r="EZ39">
         <v>0.26139994191113403</v>
@@ -42383,10 +42629,13 @@
       <c r="FB39">
         <v>0.119083060434663</v>
       </c>
+      <c r="FC39">
+        <v>8.7438064704154606E-2</v>
+      </c>
     </row>
-    <row r="40" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B40">
         <v>1.6172506738544501</v>
@@ -42848,7 +43097,7 @@
         <v>-0.25706940874036399</v>
       </c>
       <c r="EY40">
-        <v>-0.248138957816363</v>
+        <v>0</v>
       </c>
       <c r="EZ40">
         <v>0.49382716049383402</v>
@@ -42859,10 +43108,13 @@
       <c r="FB40">
         <v>1.5228426395939101</v>
       </c>
+      <c r="FC40">
+        <v>1.4814814814814801</v>
+      </c>
     </row>
-    <row r="41" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B41">
         <v>1.9471859162443399</v>
@@ -43324,7 +43576,7 @@
         <v>0.44490970950011299</v>
       </c>
       <c r="EY41">
-        <v>0.30112923462987301</v>
+        <v>0</v>
       </c>
       <c r="EZ41">
         <v>0.198955483710508</v>
@@ -43333,12 +43585,15 @@
         <v>1.74224955162696</v>
       </c>
       <c r="FB41">
-        <v>0.51719679337989599</v>
+        <v>0.232738557020955</v>
+      </c>
+      <c r="FC41">
+        <v>-0.90135202804205505</v>
       </c>
     </row>
-    <row r="42" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B42">
         <v>0.749829584185428</v>
@@ -43800,7 +44055,7 @@
         <v>1.31492439184745</v>
       </c>
       <c r="EY42">
-        <v>1.2171684817424799</v>
+        <v>0</v>
       </c>
       <c r="EZ42">
         <v>1.1450381679389401</v>
@@ -43811,10 +44066,13 @@
       <c r="FB42">
         <v>1.5688949522510101</v>
       </c>
+      <c r="FC42">
+        <v>1.4193548387096699</v>
+      </c>
     </row>
-    <row r="43" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B43">
         <v>-0.38372985418265498</v>
@@ -44276,7 +44534,7 @@
         <v>0.78802206461780899</v>
       </c>
       <c r="EY43">
-        <v>-0.99999999999998401</v>
+        <v>0</v>
       </c>
       <c r="EZ43">
         <v>-1.55038759689922</v>
@@ -44287,10 +44545,13 @@
       <c r="FB43">
         <v>-2.1428571428571401</v>
       </c>
+      <c r="FC43">
+        <v>-2.2456140350877098</v>
+      </c>
     </row>
-    <row r="44" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B44">
         <v>-0.72695551032275196</v>
@@ -44752,7 +45013,7 @@
         <v>0.66686874810546604</v>
       </c>
       <c r="EY44">
-        <v>0.85900473933648602</v>
+        <v>0</v>
       </c>
       <c r="EZ44">
         <v>0.58445353594389204</v>
@@ -44763,10 +45024,13 @@
       <c r="FB44">
         <v>0.33700980392157598</v>
       </c>
+      <c r="FC44">
+        <v>0.385756676557867</v>
+      </c>
     </row>
-    <row r="45" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B45">
         <v>0.63897763578274502</v>
@@ -45228,7 +45492,7 @@
         <v>-1.0238907849829399</v>
       </c>
       <c r="EY45">
-        <v>-1.34228187919464</v>
+        <v>0</v>
       </c>
       <c r="EZ45">
         <v>-0.66006600660065795</v>
@@ -45239,10 +45503,13 @@
       <c r="FB45">
         <v>-0.342465753424675</v>
       </c>
+      <c r="FC45">
+        <v>-1.17639525788096E-14</v>
+      </c>
     </row>
-    <row r="46" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B46">
         <v>0.81709616593336398</v>
@@ -45704,7 +45971,7 @@
         <v>3.33723653395784</v>
       </c>
       <c r="EY46">
-        <v>3.2539221382916699</v>
+        <v>0</v>
       </c>
       <c r="EZ46">
         <v>3.11418685121108</v>
@@ -45715,10 +45982,13 @@
       <c r="FB46">
         <v>2.7695934001178699</v>
       </c>
+      <c r="FC46">
+        <v>2.5951557093425599</v>
+      </c>
     </row>
-    <row r="47" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B47">
         <v>0</v>
@@ -46180,7 +46450,7 @@
         <v>0.53191489361702904</v>
       </c>
       <c r="EY47">
-        <v>-0.25641025641026</v>
+        <v>0</v>
       </c>
       <c r="EZ47">
         <v>-1.01265822784812</v>
@@ -46191,10 +46461,13 @@
       <c r="FB47">
         <v>-0.26737967914440802</v>
       </c>
+      <c r="FC47">
+        <v>-0.76726342710998496</v>
+      </c>
     </row>
-    <row r="48" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B48">
         <v>-0.92449922958396702</v>
@@ -46656,7 +46929,7 @@
         <v>2.97077144226163</v>
       </c>
       <c r="EY48">
-        <v>2.5581395348837201</v>
+        <v>0</v>
       </c>
       <c r="EZ48">
         <v>2.6802218114602598</v>
@@ -46667,10 +46940,13 @@
       <c r="FB48">
         <v>2.35872235872236</v>
       </c>
+      <c r="FC48">
+        <v>2.7505827505827498</v>
+      </c>
     </row>
-    <row r="49" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B49">
         <v>0.55447470817121103</v>
@@ -47132,7 +47408,7 @@
         <v>0.60384419118898902</v>
       </c>
       <c r="EY49">
-        <v>0.71859254976460296</v>
+        <v>0</v>
       </c>
       <c r="EZ49">
         <v>0.44204322200393698</v>
@@ -47141,12 +47417,15 @@
         <v>0.91546391752576595</v>
       </c>
       <c r="FB49">
-        <v>0.36201380703821801</v>
+        <v>0.202054217881806</v>
+      </c>
+      <c r="FC49">
+        <v>0.37073652990608003</v>
       </c>
     </row>
-    <row r="50" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B50">
         <v>1.9178082191780801</v>
@@ -47608,7 +47887,7 @@
         <v>0.99009900990097699</v>
       </c>
       <c r="EY50">
-        <v>0.96654275092937603</v>
+        <v>0</v>
       </c>
       <c r="EZ50">
         <v>0.88495575221238099</v>
@@ -47619,10 +47898,13 @@
       <c r="FB50">
         <v>0.60286360211003098</v>
       </c>
+      <c r="FC50">
+        <v>0.58953574060428304</v>
+      </c>
     </row>
-    <row r="51" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B51">
         <v>1.8181818181818199</v>
@@ -48084,7 +48366,7 @@
         <v>0.31948881789136702</v>
       </c>
       <c r="EY51">
-        <v>0.30674846625767299</v>
+        <v>0</v>
       </c>
       <c r="EZ51">
         <v>0.30303030303030698</v>
@@ -48093,12 +48375,15 @@
         <v>0.62111801242234699</v>
       </c>
       <c r="FB51">
-        <v>0.96463022508038798</v>
+        <v>0.321543408360145</v>
+      </c>
+      <c r="FC51">
+        <v>-0.30211480362538201</v>
       </c>
     </row>
-    <row r="52" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B52">
         <v>-0.80256821829855496</v>
@@ -48560,7 +48845,7 @@
         <v>2.6516306004266998</v>
       </c>
       <c r="EY52">
-        <v>3.4513537637607898</v>
+        <v>0</v>
       </c>
       <c r="EZ52">
         <v>4.6477205447010199</v>
@@ -48569,12 +48854,15 @@
         <v>2.7744982290436799</v>
       </c>
       <c r="FB52">
-        <v>2.5444512568975899</v>
+        <v>2.5751072961373298</v>
+      </c>
+      <c r="FC52">
+        <v>3.28734957440563</v>
       </c>
     </row>
-    <row r="53" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B53">
         <v>1.9118869492934201</v>
@@ -49036,7 +49324,7 @@
         <v>-4.0420371867418897E-2</v>
       </c>
       <c r="EY53">
-        <v>-0.72133637053909505</v>
+        <v>0</v>
       </c>
       <c r="EZ53">
         <v>-0.70789865871832203</v>
@@ -49047,10 +49335,13 @@
       <c r="FB53">
         <v>-0.33860045146728102</v>
       </c>
+      <c r="FC53">
+        <v>-0.37257824143070001</v>
+      </c>
     </row>
-    <row r="54" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B54">
         <v>-0.290275761973879</v>
@@ -49512,7 +49803,7 @@
         <v>-0.49261083743843098</v>
       </c>
       <c r="EY54">
-        <v>-0.63291139240507199</v>
+        <v>0</v>
       </c>
       <c r="EZ54">
         <v>-0.62500000000000899</v>
@@ -49523,10 +49814,13 @@
       <c r="FB54">
         <v>-0.17035775127769801</v>
       </c>
+      <c r="FC54">
+        <v>-1.1199999999999899</v>
+      </c>
     </row>
-    <row r="55" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B55">
         <v>-0.75301204819277101</v>
@@ -49988,7 +50282,7 @@
         <v>-0.58394160583941102</v>
       </c>
       <c r="EY55">
-        <v>-1.86046511627907</v>
+        <v>0</v>
       </c>
       <c r="EZ55">
         <v>-1.3876040703052701</v>
@@ -49997,12 +50291,15 @@
         <v>-0.14157621519583899</v>
       </c>
       <c r="FB55">
-        <v>-2.15053763440861</v>
+        <v>-2.1994134897360702</v>
+      </c>
+      <c r="FC55">
+        <v>-1.8621973929236399</v>
       </c>
     </row>
-    <row r="56" spans="1:158" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:159" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B56">
         <v>0.95541401273885596</v>
@@ -50464,7 +50761,7 @@
         <v>0.334448160535122</v>
       </c>
       <c r="EY56">
-        <v>0.970873786407769</v>
+        <v>0</v>
       </c>
       <c r="EZ56">
         <v>0</v>
@@ -50474,6 +50771,9 @@
       </c>
       <c r="FB56">
         <v>-1.6949152542372901</v>
+      </c>
+      <c r="FC56">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
SEM update May 22 2026
</commit_message>
<xml_diff>
--- a/static/data/source/state_and_local_public_education_employment.xlsx
+++ b/static/data/source/state_and_local_public_education_employment.xlsx
@@ -370,7 +370,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A4:FP56"/>
+  <dimension ref="A4:FQ56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="4">
@@ -1234,6 +1234,11 @@
           <t>03/01/2026</t>
         </is>
       </c>
+      <c r="FQ4" t="inlineStr">
+        <is>
+          <t>04/01/2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1749,10 +1754,13 @@
         <v>10913.3</v>
       </c>
       <c r="FO5">
-        <v>11238.1</v>
+        <v>11224.6</v>
       </c>
       <c r="FP5">
-        <v>11294.4</v>
+        <v>11276.4</v>
+      </c>
+      <c r="FQ5">
+        <v>11247.4</v>
       </c>
     </row>
     <row r="6">
@@ -2272,7 +2280,10 @@
         <v>185.4</v>
       </c>
       <c r="FP6">
-        <v>186.3</v>
+        <v>186.6</v>
+      </c>
+      <c r="FQ6">
+        <v>185.9</v>
       </c>
     </row>
     <row r="7">
@@ -2794,6 +2805,9 @@
       <c r="FP7">
         <v>27.9</v>
       </c>
+      <c r="FQ7">
+        <v>27.9</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3314,6 +3328,9 @@
       <c r="FP8">
         <v>198.6</v>
       </c>
+      <c r="FQ8">
+        <v>200.5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3834,6 +3851,9 @@
       <c r="FP9">
         <v>97.6</v>
       </c>
+      <c r="FQ9">
+        <v>97.4</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4352,7 +4372,10 @@
         <v>1267.8</v>
       </c>
       <c r="FP10">
-        <v>1289.6</v>
+        <v>1292.4</v>
+      </c>
+      <c r="FQ10">
+        <v>1294.6</v>
       </c>
     </row>
     <row r="11">
@@ -4874,6 +4897,9 @@
       <c r="FP11">
         <v>247.3</v>
       </c>
+      <c r="FQ11">
+        <v>246.5</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5392,7 +5418,10 @@
         <v>125.7</v>
       </c>
       <c r="FP12">
-        <v>126.4</v>
+        <v>126.5</v>
+      </c>
+      <c r="FQ12">
+        <v>126.2</v>
       </c>
     </row>
     <row r="13">
@@ -5912,7 +5941,10 @@
         <v>39.5</v>
       </c>
       <c r="FP13">
-        <v>40.6</v>
+        <v>39.7</v>
+      </c>
+      <c r="FQ13">
+        <v>39.6</v>
       </c>
     </row>
     <row r="14">
@@ -6434,6 +6466,9 @@
       <c r="FP14" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FQ14" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6954,6 +6989,9 @@
       <c r="FP15">
         <v>501.1</v>
       </c>
+      <c r="FQ15">
+        <v>500.2</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -7474,6 +7512,9 @@
       <c r="FP16">
         <v>355.1</v>
       </c>
+      <c r="FQ16">
+        <v>354</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -7994,6 +8035,9 @@
       <c r="FP17" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FQ17" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -8514,6 +8558,9 @@
       <c r="FP18">
         <v>64.4</v>
       </c>
+      <c r="FQ18">
+        <v>64</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -9034,6 +9081,9 @@
       <c r="FP19">
         <v>473.5</v>
       </c>
+      <c r="FQ19">
+        <v>471</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -9552,7 +9602,10 @@
         <v>228</v>
       </c>
       <c r="FP20">
-        <v>229.5</v>
+        <v>229.3</v>
+      </c>
+      <c r="FQ20">
+        <v>227.1</v>
       </c>
     </row>
     <row r="21">
@@ -10072,7 +10125,10 @@
         <v>150.5</v>
       </c>
       <c r="FP21">
-        <v>150.3</v>
+        <v>150.2</v>
+      </c>
+      <c r="FQ21">
+        <v>150</v>
       </c>
     </row>
     <row r="22">
@@ -10594,6 +10650,9 @@
       <c r="FP22">
         <v>140.2</v>
       </c>
+      <c r="FQ22">
+        <v>140.4</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -11112,7 +11171,10 @@
         <v>163.9</v>
       </c>
       <c r="FP23">
-        <v>166.6</v>
+        <v>166.5</v>
+      </c>
+      <c r="FQ23">
+        <v>165.7</v>
       </c>
     </row>
     <row r="24">
@@ -11634,6 +11696,9 @@
       <c r="FP24">
         <v>152.1</v>
       </c>
+      <c r="FQ24">
+        <v>153</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -12152,6 +12217,9 @@
         <v>49.1</v>
       </c>
       <c r="FP25">
+        <v>49.3</v>
+      </c>
+      <c r="FQ25">
         <v>49.2</v>
       </c>
     </row>
@@ -12674,6 +12742,9 @@
       <c r="FP26">
         <v>231.8</v>
       </c>
+      <c r="FQ26">
+        <v>230.7</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -13194,6 +13265,9 @@
       <c r="FP27">
         <v>250.8</v>
       </c>
+      <c r="FQ27">
+        <v>251.5</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -13714,6 +13788,9 @@
       <c r="FP28">
         <v>335.3</v>
       </c>
+      <c r="FQ28">
+        <v>333.5</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -14234,6 +14311,9 @@
       <c r="FP29">
         <v>217.2</v>
       </c>
+      <c r="FQ29">
+        <v>220.3</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -14754,6 +14834,9 @@
       <c r="FP30">
         <v>104.8</v>
       </c>
+      <c r="FQ30">
+        <v>104.4</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -15274,6 +15357,9 @@
       <c r="FP31" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FQ31" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -15794,6 +15880,9 @@
       <c r="FP32">
         <v>42.4</v>
       </c>
+      <c r="FQ32">
+        <v>42.8</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -16312,7 +16401,10 @@
         <v>97.5</v>
       </c>
       <c r="FP33">
-        <v>97.8</v>
+        <v>97.7</v>
+      </c>
+      <c r="FQ33">
+        <v>98</v>
       </c>
     </row>
     <row r="34">
@@ -16834,6 +16926,9 @@
       <c r="FP34">
         <v>89.8</v>
       </c>
+      <c r="FQ34">
+        <v>89.2</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -17352,7 +17447,10 @@
         <v>43.9</v>
       </c>
       <c r="FP35">
-        <v>44</v>
+        <v>43.8</v>
+      </c>
+      <c r="FQ35">
+        <v>43.3</v>
       </c>
     </row>
     <row r="36">
@@ -17872,7 +17970,10 @@
         <v>337.7</v>
       </c>
       <c r="FP36">
-        <v>338.6</v>
+        <v>338.7</v>
+      </c>
+      <c r="FQ36">
+        <v>340.3</v>
       </c>
     </row>
     <row r="37">
@@ -18394,6 +18495,9 @@
       <c r="FP37">
         <v>80.7</v>
       </c>
+      <c r="FQ37">
+        <v>79.8</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -18912,7 +19016,10 @@
         <v>700.7</v>
       </c>
       <c r="FP38">
-        <v>704.4</v>
+        <v>701.5</v>
+      </c>
+      <c r="FQ38">
+        <v>698.6</v>
       </c>
     </row>
     <row r="39">
@@ -19434,6 +19541,9 @@
       <c r="FP39">
         <v>343.7</v>
       </c>
+      <c r="FQ39">
+        <v>348.5</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -19954,6 +20064,9 @@
       <c r="FP40">
         <v>41.2</v>
       </c>
+      <c r="FQ40">
+        <v>40.9</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -20472,7 +20585,10 @@
         <v>395.8</v>
       </c>
       <c r="FP41">
-        <v>401.1</v>
+        <v>400</v>
+      </c>
+      <c r="FQ41">
+        <v>396.7</v>
       </c>
     </row>
     <row r="42">
@@ -20994,6 +21110,9 @@
       <c r="FP42">
         <v>158.3</v>
       </c>
+      <c r="FQ42">
+        <v>159</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -21514,6 +21633,9 @@
       <c r="FP43">
         <v>139.2</v>
       </c>
+      <c r="FQ43">
+        <v>138.9</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -22032,7 +22154,10 @@
         <v>338.3</v>
       </c>
       <c r="FP44">
-        <v>340.2</v>
+        <v>340.1</v>
+      </c>
+      <c r="FQ44">
+        <v>340.4</v>
       </c>
     </row>
     <row r="45">
@@ -22554,6 +22679,9 @@
       <c r="FP45">
         <v>30.3</v>
       </c>
+      <c r="FQ45">
+        <v>30</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -23074,6 +23202,9 @@
       <c r="FP46">
         <v>178</v>
       </c>
+      <c r="FQ46">
+        <v>176.7</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -23594,6 +23725,9 @@
       <c r="FP47">
         <v>39.1</v>
       </c>
+      <c r="FQ47">
+        <v>38.8</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -24114,6 +24248,9 @@
       <c r="FP48">
         <v>220.4</v>
       </c>
+      <c r="FQ48">
+        <v>218.2</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -24634,6 +24771,9 @@
       <c r="FP49">
         <v>1223.5</v>
       </c>
+      <c r="FQ49">
+        <v>1219.7</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -25154,6 +25294,9 @@
       <c r="FP50">
         <v>136.3</v>
       </c>
+      <c r="FQ50">
+        <v>136.1</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -25672,7 +25815,10 @@
         <v>33</v>
       </c>
       <c r="FP51">
-        <v>32.9</v>
+        <v>33.1</v>
+      </c>
+      <c r="FQ51">
+        <v>32.6</v>
       </c>
     </row>
     <row r="52">
@@ -26192,7 +26338,10 @@
         <v>351.9</v>
       </c>
       <c r="FP52">
-        <v>353.7</v>
+        <v>353.5</v>
+      </c>
+      <c r="FQ52">
+        <v>353.3</v>
       </c>
     </row>
     <row r="53">
@@ -26712,7 +26861,10 @@
         <v>267.4</v>
       </c>
       <c r="FP53">
-        <v>268.1</v>
+        <v>267.9</v>
+      </c>
+      <c r="FQ53">
+        <v>267.2</v>
       </c>
     </row>
     <row r="54">
@@ -27232,7 +27384,10 @@
         <v>61.8</v>
       </c>
       <c r="FP54">
-        <v>62.9</v>
+        <v>63</v>
+      </c>
+      <c r="FQ54">
+        <v>62.6</v>
       </c>
     </row>
     <row r="55">
@@ -27754,6 +27909,9 @@
       <c r="FP55">
         <v>210.8</v>
       </c>
+      <c r="FQ55">
+        <v>210.7</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -28273,6 +28431,9 @@
       </c>
       <c r="FP56">
         <v>31.6</v>
+      </c>
+      <c r="FQ56">
+        <v>31.4</v>
       </c>
     </row>
   </sheetData>
@@ -28284,7 +28445,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A4:FD56"/>
+  <dimension ref="A4:FE56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="4">
@@ -29088,6 +29249,11 @@
           <t>03/01/2026</t>
         </is>
       </c>
+      <c r="FE4" t="inlineStr">
+        <is>
+          <t>04/01/2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -29567,10 +29733,13 @@
         <v>0.0192462790527031</v>
       </c>
       <c r="FC5">
-        <v>-0.0133456706644365</v>
+        <v>-0.133456706644381</v>
       </c>
       <c r="FD5">
-        <v>0.0877309583942544</v>
+        <v>-0.0717798750498504</v>
+      </c>
+      <c r="FE5">
+        <v>-0.270440418872292</v>
       </c>
     </row>
     <row r="6">
@@ -30054,7 +30223,10 @@
         <v>3</v>
       </c>
       <c r="FD6">
-        <v>2.87134180011043</v>
+        <v>3.03699613473218</v>
+      </c>
+      <c r="FE6">
+        <v>3.16315205327413</v>
       </c>
     </row>
     <row r="7">
@@ -30540,6 +30712,9 @@
       <c r="FD7">
         <v>-3.12500000000001</v>
       </c>
+      <c r="FE7">
+        <v>-2.78745644599303</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -31024,6 +31199,9 @@
       <c r="FD8">
         <v>-2.45579567779961</v>
       </c>
+      <c r="FE8">
+        <v>-2.57531584062195</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -31508,6 +31686,9 @@
       <c r="FD9">
         <v>-0.102354145342895</v>
       </c>
+      <c r="FE9">
+        <v>-0.510725229826353</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -31990,7 +32171,10 @@
         <v>-1.83507549361208</v>
       </c>
       <c r="FD10">
-        <v>-2.08792043125047</v>
+        <v>-1.87533216915952</v>
+      </c>
+      <c r="FE10">
+        <v>-2.10223835450697</v>
       </c>
     </row>
     <row r="11">
@@ -32476,6 +32660,9 @@
       <c r="FD11">
         <v>1.3940139401394</v>
       </c>
+      <c r="FE11">
+        <v>1.77539223781999</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -32958,7 +33145,10 @@
         <v>-0.238095238095236</v>
       </c>
       <c r="FD12">
-        <v>-0.315457413249205</v>
+        <v>-0.236593059936906</v>
+      </c>
+      <c r="FE12">
+        <v>-0.473186119873813</v>
       </c>
     </row>
     <row r="13">
@@ -33442,7 +33632,10 @@
         <v>1.54241645244216</v>
       </c>
       <c r="FD13">
-        <v>0.995024875621887</v>
+        <v>-1.24378109452736</v>
+      </c>
+      <c r="FE13">
+        <v>-1.98019801980197</v>
       </c>
     </row>
     <row r="14">
@@ -33928,6 +34121,9 @@
       <c r="FD14" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FE14" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -34412,6 +34608,9 @@
       <c r="FD15">
         <v>-1.20268138801261</v>
       </c>
+      <c r="FE15">
+        <v>-1.04846686449059</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -34896,6 +35095,9 @@
       <c r="FD16">
         <v>0.766174801362101</v>
       </c>
+      <c r="FE16">
+        <v>0.53961942629934</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -35380,6 +35582,9 @@
       <c r="FD17" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FE17" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -35864,6 +36069,9 @@
       <c r="FD18">
         <v>-0.155038759689914</v>
       </c>
+      <c r="FE18">
+        <v>-0.311526479750783</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -36348,6 +36556,9 @@
       <c r="FD19">
         <v>1.13199487398547</v>
       </c>
+      <c r="FE19">
+        <v>1.00793480591893</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -36830,7 +37041,10 @@
         <v>-1.68175937904268</v>
       </c>
       <c r="FD20">
-        <v>-4.3351396415173</v>
+        <v>-4.41850771154648</v>
+      </c>
+      <c r="FE20">
+        <v>-6.07940446650125</v>
       </c>
     </row>
     <row r="21">
@@ -37314,7 +37528,10 @@
         <v>-0.265076209410209</v>
       </c>
       <c r="FD21">
-        <v>0.200000000000008</v>
+        <v>0.133333333333326</v>
+      </c>
+      <c r="FE21">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -37800,6 +38017,9 @@
       <c r="FD22">
         <v>0.790797987059665</v>
       </c>
+      <c r="FE22">
+        <v>0.645161290322585</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -38282,7 +38502,10 @@
         <v>-1.145958986731</v>
       </c>
       <c r="FD23">
-        <v>-0.0599880023995167</v>
+        <v>-0.119976004799033</v>
+      </c>
+      <c r="FE23">
+        <v>-0.180722891566272</v>
       </c>
     </row>
     <row r="24">
@@ -38768,6 +38991,9 @@
       <c r="FD24">
         <v>-0.0657030223390239</v>
       </c>
+      <c r="FE24">
+        <v>-0.0653167864141233</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -39250,7 +39476,10 @@
         <v>-0.80808080808082</v>
       </c>
       <c r="FD25">
-        <v>-1.00603621730382</v>
+        <v>-0.80482897384307</v>
+      </c>
+      <c r="FE25">
+        <v>-1.60000000000001</v>
       </c>
     </row>
     <row r="26">
@@ -39736,6 +39965,9 @@
       <c r="FD26">
         <v>0.563991323210417</v>
       </c>
+      <c r="FE26">
+        <v>0.566695727986043</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -40220,6 +40452,9 @@
       <c r="FD27">
         <v>0.239808153477216</v>
       </c>
+      <c r="FE27">
+        <v>0.359138068635266</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -40704,6 +40939,9 @@
       <c r="FD28">
         <v>2.63238445056626</v>
       </c>
+      <c r="FE28">
+        <v>2.90033940141931</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -41188,6 +41426,9 @@
       <c r="FD29">
         <v>0.695410292072323</v>
       </c>
+      <c r="FE29">
+        <v>0.869963369963373</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -41672,6 +41913,9 @@
       <c r="FD30">
         <v>0.383141762452099</v>
       </c>
+      <c r="FE30">
+        <v>0.38461538461539</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -42156,6 +42400,9 @@
       <c r="FD31" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FE31" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -42640,6 +42887,9 @@
       <c r="FD32">
         <v>-1.39534883720931</v>
       </c>
+      <c r="FE32">
+        <v>-1.15473441108545</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -43122,7 +43372,10 @@
         <v>0.827300930713544</v>
       </c>
       <c r="FD33">
-        <v>1.24223602484472</v>
+        <v>1.13871635610767</v>
+      </c>
+      <c r="FE33">
+        <v>1.23966942148761</v>
       </c>
     </row>
     <row r="34">
@@ -43608,6 +43861,9 @@
       <c r="FD34">
         <v>0.447427293064867</v>
       </c>
+      <c r="FE34">
+        <v>-0.335195530726254</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -44090,7 +44346,10 @@
         <v>-3.30396475770925</v>
       </c>
       <c r="FD35">
-        <v>-3.2967032967033</v>
+        <v>-3.73626373626374</v>
+      </c>
+      <c r="FE35">
+        <v>-3.77777777777778</v>
       </c>
     </row>
     <row r="36">
@@ -44574,7 +44833,10 @@
         <v>0.26722090261282</v>
       </c>
       <c r="FD36">
-        <v>0.236826524570755</v>
+        <v>0.266429840142089</v>
+      </c>
+      <c r="FE36">
+        <v>0.472394449365193</v>
       </c>
     </row>
     <row r="37">
@@ -45060,6 +45322,9 @@
       <c r="FD37">
         <v>-0.981595092024536</v>
       </c>
+      <c r="FE37">
+        <v>-1.96560196560198</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -45542,7 +45807,10 @@
         <v>2.02387885847408</v>
       </c>
       <c r="FD38">
-        <v>2.05737467400754</v>
+        <v>1.63720660678065</v>
+      </c>
+      <c r="FE38">
+        <v>0.880866425992767</v>
       </c>
     </row>
     <row r="39">
@@ -46028,6 +46296,9 @@
       <c r="FD39">
         <v>0.0873616773442249</v>
       </c>
+      <c r="FE39">
+        <v>0.0861573808156265</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -46512,6 +46783,9 @@
       <c r="FD40">
         <v>1.47783251231527</v>
       </c>
+      <c r="FE40">
+        <v>1.48883374689827</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -46994,7 +47268,10 @@
         <v>-0.901352028042055</v>
       </c>
       <c r="FD41">
-        <v>1.51860288534548</v>
+        <v>1.24019235636547</v>
+      </c>
+      <c r="FE41">
+        <v>-0.576441102756895</v>
       </c>
     </row>
     <row r="42">
@@ -47480,6 +47757,9 @@
       <c r="FD42">
         <v>1.40935297885972</v>
       </c>
+      <c r="FE42">
+        <v>1.27388535031847</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -47964,6 +48244,9 @@
       <c r="FD43">
         <v>-2.72536687631028</v>
       </c>
+      <c r="FE43">
+        <v>-2.32067510548524</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -48446,7 +48729,10 @@
         <v>0.385756676557867</v>
       </c>
       <c r="FD44">
-        <v>0.383593980525232</v>
+        <v>0.354086751254054</v>
+      </c>
+      <c r="FE44">
+        <v>0.383367738130332</v>
       </c>
     </row>
     <row r="45">
@@ -48932,6 +49218,9 @@
       <c r="FD45">
         <v>-0.328947368421057</v>
       </c>
+      <c r="FE45">
+        <v>-0.662251655629137</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -49416,6 +49705,9 @@
       <c r="FD46">
         <v>2.71206001154067</v>
       </c>
+      <c r="FE46">
+        <v>2.13872832369942</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -49900,6 +50192,9 @@
       <c r="FD47">
         <v>-0.25510204081633</v>
       </c>
+      <c r="FE47">
+        <v>-0.767263427109985</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -50384,6 +50679,9 @@
       <c r="FD48">
         <v>2.60707635009312</v>
       </c>
+      <c r="FE48">
+        <v>2.15355805243447</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -50868,6 +51166,9 @@
       <c r="FD49">
         <v>0.674730519213367</v>
       </c>
+      <c r="FE49">
+        <v>0.710098257782174</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -51352,6 +51653,9 @@
       <c r="FD50">
         <v>0.516224188790573</v>
       </c>
+      <c r="FE50">
+        <v>0.591278640059115</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -51834,7 +52138,10 @@
         <v>-0.302114803625382</v>
       </c>
       <c r="FD51">
-        <v>-0.303030303030307</v>
+        <v>0.303030303030307</v>
+      </c>
+      <c r="FE51">
+        <v>-1.80722891566265</v>
       </c>
     </row>
     <row r="52">
@@ -52318,7 +52625,10 @@
         <v>3.28734957440563</v>
       </c>
       <c r="FD52">
-        <v>3.27007299270073</v>
+        <v>3.21167883211679</v>
+      </c>
+      <c r="FE52">
+        <v>2.76323443862713</v>
       </c>
     </row>
     <row r="53">
@@ -52802,7 +53112,10 @@
         <v>-0.3725782414307</v>
       </c>
       <c r="FD53">
-        <v>-0.556379821958457</v>
+        <v>-0.630563798219601</v>
+      </c>
+      <c r="FE53">
+        <v>-0.890207715133523</v>
       </c>
     </row>
     <row r="54">
@@ -53286,7 +53599,10 @@
         <v>-1.11999999999999</v>
       </c>
       <c r="FD54">
-        <v>-0.474683544303793</v>
+        <v>-0.316455696202536</v>
+      </c>
+      <c r="FE54">
+        <v>-1.57232704402515</v>
       </c>
     </row>
     <row r="55">
@@ -53772,6 +54088,9 @@
       <c r="FD55">
         <v>-1.86219739292364</v>
       </c>
+      <c r="FE55">
+        <v>-2.22737819025523</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -54255,6 +54574,9 @@
       </c>
       <c r="FD56">
         <v>0.317460317460311</v>
+      </c>
+      <c r="FE56">
+        <v>0.319488817891367</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
SEM Update on June 23, 2026
</commit_message>
<xml_diff>
--- a/static/data/source/state_and_local_public_education_employment.xlsx
+++ b/static/data/source/state_and_local_public_education_employment.xlsx
@@ -370,7 +370,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A4:FQ56"/>
+  <dimension ref="A4:FR56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="4">
@@ -1239,6 +1239,11 @@
           <t>04/01/2026</t>
         </is>
       </c>
+      <c r="FR4" t="inlineStr">
+        <is>
+          <t>05/01/2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1757,10 +1762,13 @@
         <v>11224.6</v>
       </c>
       <c r="FP5">
-        <v>11276.4</v>
+        <v>11275.1</v>
       </c>
       <c r="FQ5">
-        <v>11247.4</v>
+        <v>11248.4</v>
+      </c>
+      <c r="FR5">
+        <v>11095</v>
       </c>
     </row>
     <row r="6">
@@ -2285,6 +2293,9 @@
       <c r="FQ6">
         <v>185.9</v>
       </c>
+      <c r="FR6">
+        <v>186</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2808,6 +2819,9 @@
       <c r="FQ7">
         <v>27.9</v>
       </c>
+      <c r="FR7">
+        <v>27</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3329,7 +3343,10 @@
         <v>198.6</v>
       </c>
       <c r="FQ8">
-        <v>200.5</v>
+        <v>200.6</v>
+      </c>
+      <c r="FR8">
+        <v>188</v>
       </c>
     </row>
     <row r="9">
@@ -3854,6 +3871,9 @@
       <c r="FQ9">
         <v>97.4</v>
       </c>
+      <c r="FR9">
+        <v>97.1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4375,7 +4395,10 @@
         <v>1292.4</v>
       </c>
       <c r="FQ10">
-        <v>1294.6</v>
+        <v>1295</v>
+      </c>
+      <c r="FR10">
+        <v>1300.7</v>
       </c>
     </row>
     <row r="11">
@@ -4898,7 +4921,10 @@
         <v>247.3</v>
       </c>
       <c r="FQ11">
-        <v>246.5</v>
+        <v>246.4</v>
+      </c>
+      <c r="FR11">
+        <v>246.3</v>
       </c>
     </row>
     <row r="12">
@@ -5421,7 +5447,10 @@
         <v>126.5</v>
       </c>
       <c r="FQ12">
-        <v>126.2</v>
+        <v>125</v>
+      </c>
+      <c r="FR12">
+        <v>124.4</v>
       </c>
     </row>
     <row r="13">
@@ -5944,7 +5973,10 @@
         <v>39.7</v>
       </c>
       <c r="FQ13">
-        <v>39.6</v>
+        <v>39.4</v>
+      </c>
+      <c r="FR13">
+        <v>38.7</v>
       </c>
     </row>
     <row r="14">
@@ -6469,6 +6501,9 @@
       <c r="FQ14" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FR14" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6990,7 +7025,10 @@
         <v>501.1</v>
       </c>
       <c r="FQ15">
-        <v>500.2</v>
+        <v>500.4</v>
+      </c>
+      <c r="FR15">
+        <v>485.4</v>
       </c>
     </row>
     <row r="16">
@@ -7513,7 +7551,10 @@
         <v>355.1</v>
       </c>
       <c r="FQ16">
-        <v>354</v>
+        <v>353.9</v>
+      </c>
+      <c r="FR16">
+        <v>351.5</v>
       </c>
     </row>
     <row r="17">
@@ -8038,6 +8079,9 @@
       <c r="FQ17" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FR17" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -8561,6 +8605,9 @@
       <c r="FQ18">
         <v>64</v>
       </c>
+      <c r="FR18">
+        <v>61.8</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -9082,7 +9129,10 @@
         <v>473.5</v>
       </c>
       <c r="FQ19">
-        <v>471</v>
+        <v>470.8</v>
+      </c>
+      <c r="FR19">
+        <v>467</v>
       </c>
     </row>
     <row r="20">
@@ -9605,7 +9655,10 @@
         <v>229.3</v>
       </c>
       <c r="FQ20">
-        <v>227.1</v>
+        <v>227.3</v>
+      </c>
+      <c r="FR20">
+        <v>222.8</v>
       </c>
     </row>
     <row r="21">
@@ -10128,7 +10181,10 @@
         <v>150.2</v>
       </c>
       <c r="FQ21">
-        <v>150</v>
+        <v>149.8</v>
+      </c>
+      <c r="FR21">
+        <v>150.1</v>
       </c>
     </row>
     <row r="22">
@@ -10653,6 +10709,9 @@
       <c r="FQ22">
         <v>140.4</v>
       </c>
+      <c r="FR22">
+        <v>137.4</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -11176,6 +11235,9 @@
       <c r="FQ23">
         <v>165.7</v>
       </c>
+      <c r="FR23">
+        <v>165.8</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -11699,6 +11761,9 @@
       <c r="FQ24">
         <v>153</v>
       </c>
+      <c r="FR24">
+        <v>151.9</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -12220,6 +12285,9 @@
         <v>49.3</v>
       </c>
       <c r="FQ25">
+        <v>49.1</v>
+      </c>
+      <c r="FR25">
         <v>49.2</v>
       </c>
     </row>
@@ -12745,6 +12813,9 @@
       <c r="FQ26">
         <v>230.7</v>
       </c>
+      <c r="FR26">
+        <v>230.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -13268,6 +13339,9 @@
       <c r="FQ27">
         <v>251.5</v>
       </c>
+      <c r="FR27">
+        <v>251.5</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -13791,6 +13865,9 @@
       <c r="FQ28">
         <v>333.5</v>
       </c>
+      <c r="FR28">
+        <v>319.7</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -14314,6 +14391,9 @@
       <c r="FQ29">
         <v>220.3</v>
       </c>
+      <c r="FR29">
+        <v>217.3</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -14837,6 +14917,9 @@
       <c r="FQ30">
         <v>104.4</v>
       </c>
+      <c r="FR30">
+        <v>103.3</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -15360,6 +15443,9 @@
       <c r="FQ31" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FR31" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -15883,6 +15969,9 @@
       <c r="FQ32">
         <v>42.8</v>
       </c>
+      <c r="FR32">
+        <v>43.4</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -16406,6 +16495,9 @@
       <c r="FQ33">
         <v>98</v>
       </c>
+      <c r="FR33">
+        <v>97.8</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -16927,7 +17019,10 @@
         <v>89.8</v>
       </c>
       <c r="FQ34">
-        <v>89.2</v>
+        <v>89.1</v>
+      </c>
+      <c r="FR34">
+        <v>89.5</v>
       </c>
     </row>
     <row r="35">
@@ -17450,7 +17545,10 @@
         <v>43.8</v>
       </c>
       <c r="FQ35">
-        <v>43.3</v>
+        <v>43.9</v>
+      </c>
+      <c r="FR35">
+        <v>42.3</v>
       </c>
     </row>
     <row r="36">
@@ -17973,7 +18071,10 @@
         <v>338.7</v>
       </c>
       <c r="FQ36">
-        <v>340.3</v>
+        <v>340.2</v>
+      </c>
+      <c r="FR36">
+        <v>335.7</v>
       </c>
     </row>
     <row r="37">
@@ -18496,7 +18597,10 @@
         <v>80.7</v>
       </c>
       <c r="FQ37">
-        <v>79.8</v>
+        <v>81.1</v>
+      </c>
+      <c r="FR37">
+        <v>80.3</v>
       </c>
     </row>
     <row r="38">
@@ -19019,7 +19123,10 @@
         <v>701.5</v>
       </c>
       <c r="FQ38">
-        <v>698.6</v>
+        <v>699.2</v>
+      </c>
+      <c r="FR38">
+        <v>697.6</v>
       </c>
     </row>
     <row r="39">
@@ -19544,6 +19651,9 @@
       <c r="FQ39">
         <v>348.5</v>
       </c>
+      <c r="FR39">
+        <v>347.3</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -20067,6 +20177,9 @@
       <c r="FQ40">
         <v>40.9</v>
       </c>
+      <c r="FR40">
+        <v>40.8</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -20588,7 +20701,10 @@
         <v>400</v>
       </c>
       <c r="FQ41">
-        <v>396.7</v>
+        <v>396.6</v>
+      </c>
+      <c r="FR41">
+        <v>385.3</v>
       </c>
     </row>
     <row r="42">
@@ -21113,6 +21229,9 @@
       <c r="FQ42">
         <v>159</v>
       </c>
+      <c r="FR42">
+        <v>158.6</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -21636,6 +21755,9 @@
       <c r="FQ43">
         <v>138.9</v>
       </c>
+      <c r="FR43">
+        <v>139.4</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -22159,6 +22281,9 @@
       <c r="FQ44">
         <v>340.4</v>
       </c>
+      <c r="FR44">
+        <v>339.1</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -22682,6 +22807,9 @@
       <c r="FQ45">
         <v>30</v>
       </c>
+      <c r="FR45">
+        <v>28.9</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -23203,7 +23331,10 @@
         <v>178</v>
       </c>
       <c r="FQ46">
-        <v>176.7</v>
+        <v>176.8</v>
+      </c>
+      <c r="FR46">
+        <v>169.8</v>
       </c>
     </row>
     <row r="47">
@@ -23728,6 +23859,9 @@
       <c r="FQ47">
         <v>38.8</v>
       </c>
+      <c r="FR47">
+        <v>38.3</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -24251,6 +24385,9 @@
       <c r="FQ48">
         <v>218.2</v>
       </c>
+      <c r="FR48">
+        <v>215</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -24772,7 +24909,10 @@
         <v>1223.5</v>
       </c>
       <c r="FQ49">
-        <v>1219.7</v>
+        <v>1221.1</v>
+      </c>
+      <c r="FR49">
+        <v>1219</v>
       </c>
     </row>
     <row r="50">
@@ -25297,6 +25437,9 @@
       <c r="FQ50">
         <v>136.1</v>
       </c>
+      <c r="FR50">
+        <v>135.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -25818,7 +25961,10 @@
         <v>33.1</v>
       </c>
       <c r="FQ51">
-        <v>32.6</v>
+        <v>32.7</v>
+      </c>
+      <c r="FR51">
+        <v>30</v>
       </c>
     </row>
     <row r="52">
@@ -26343,6 +26489,9 @@
       <c r="FQ52">
         <v>353.3</v>
       </c>
+      <c r="FR52">
+        <v>344.2</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -26864,7 +27013,10 @@
         <v>267.9</v>
       </c>
       <c r="FQ53">
-        <v>267.2</v>
+        <v>267.1</v>
+      </c>
+      <c r="FR53">
+        <v>268.8</v>
       </c>
     </row>
     <row r="54">
@@ -27389,6 +27541,9 @@
       <c r="FQ54">
         <v>62.6</v>
       </c>
+      <c r="FR54">
+        <v>62.6</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -27910,7 +28065,10 @@
         <v>210.8</v>
       </c>
       <c r="FQ55">
-        <v>210.7</v>
+        <v>210.8</v>
+      </c>
+      <c r="FR55">
+        <v>208.1</v>
       </c>
     </row>
     <row r="56">
@@ -28433,7 +28591,10 @@
         <v>31.6</v>
       </c>
       <c r="FQ56">
-        <v>31.4</v>
+        <v>31.5</v>
+      </c>
+      <c r="FR56">
+        <v>31.6</v>
       </c>
     </row>
   </sheetData>
@@ -28445,7 +28606,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A4:FE56"/>
+  <dimension ref="A4:FF56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="4">
@@ -29254,6 +29415,11 @@
           <t>04/01/2026</t>
         </is>
       </c>
+      <c r="FF4" t="inlineStr">
+        <is>
+          <t>05/01/2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -29736,10 +29902,13 @@
         <v>-0.133456706644381</v>
       </c>
       <c r="FD5">
-        <v>-0.0717798750498504</v>
+        <v>-0.083300101909712</v>
       </c>
       <c r="FE5">
-        <v>-0.270440418872292</v>
+        <v>-0.261573519892888</v>
+      </c>
+      <c r="FF5">
+        <v>-0.0603511173964413</v>
       </c>
     </row>
     <row r="6">
@@ -30228,6 +30397,9 @@
       <c r="FE6">
         <v>3.16315205327413</v>
       </c>
+      <c r="FF6">
+        <v>3.10421286031043</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -30715,6 +30887,9 @@
       <c r="FE7">
         <v>-2.78745644599303</v>
       </c>
+      <c r="FF7">
+        <v>-2.87769784172662</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -31200,7 +31375,10 @@
         <v>-2.45579567779961</v>
       </c>
       <c r="FE8">
-        <v>-2.57531584062195</v>
+        <v>-2.52672497570455</v>
+      </c>
+      <c r="FF8">
+        <v>-0.3709591944886</v>
       </c>
     </row>
     <row r="9">
@@ -31689,6 +31867,9 @@
       <c r="FE9">
         <v>-0.510725229826353</v>
       </c>
+      <c r="FF9">
+        <v>-0.614124872057313</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -32174,7 +32355,10 @@
         <v>-1.87533216915952</v>
       </c>
       <c r="FE10">
-        <v>-2.10223835450697</v>
+        <v>-2.07199032062917</v>
+      </c>
+      <c r="FF10">
+        <v>-1.75981873111784</v>
       </c>
     </row>
     <row r="11">
@@ -32661,7 +32845,10 @@
         <v>1.3940139401394</v>
       </c>
       <c r="FE11">
-        <v>1.77539223781999</v>
+        <v>1.73410404624277</v>
+      </c>
+      <c r="FF11">
+        <v>1.60891089108912</v>
       </c>
     </row>
     <row r="12">
@@ -33148,7 +33335,10 @@
         <v>-0.236593059936906</v>
       </c>
       <c r="FE12">
-        <v>-0.473186119873813</v>
+        <v>-1.41955835962145</v>
+      </c>
+      <c r="FF12">
+        <v>-1.34813639968279</v>
       </c>
     </row>
     <row r="13">
@@ -33635,7 +33825,10 @@
         <v>-1.24378109452736</v>
       </c>
       <c r="FE13">
-        <v>-1.98019801980197</v>
+        <v>-2.47524752475248</v>
+      </c>
+      <c r="FF13">
+        <v>-2.27272727272727</v>
       </c>
     </row>
     <row r="14">
@@ -34124,6 +34317,9 @@
       <c r="FE14" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FF14" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -34609,7 +34805,10 @@
         <v>-1.20268138801261</v>
       </c>
       <c r="FE15">
-        <v>-1.04846686449059</v>
+        <v>-1.00890207715134</v>
+      </c>
+      <c r="FF15">
+        <v>-1.66126418152351</v>
       </c>
     </row>
     <row r="16">
@@ -35096,7 +35295,10 @@
         <v>0.766174801362101</v>
       </c>
       <c r="FE16">
-        <v>0.53961942629934</v>
+        <v>0.511218403862542</v>
+      </c>
+      <c r="FF16">
+        <v>0.543478260869559</v>
       </c>
     </row>
     <row r="17">
@@ -35585,6 +35787,9 @@
       <c r="FE17" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FF17" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -36072,6 +36277,9 @@
       <c r="FE18">
         <v>-0.311526479750783</v>
       </c>
+      <c r="FF18">
+        <v>-1.12</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -36557,7 +36765,10 @@
         <v>1.13199487398547</v>
       </c>
       <c r="FE19">
-        <v>1.00793480591893</v>
+        <v>0.965043963113875</v>
+      </c>
+      <c r="FF19">
+        <v>0.689952565761101</v>
       </c>
     </row>
     <row r="20">
@@ -37044,7 +37255,10 @@
         <v>-4.41850771154648</v>
       </c>
       <c r="FE20">
-        <v>-6.07940446650125</v>
+        <v>-5.99669148056245</v>
+      </c>
+      <c r="FF20">
+        <v>-6.77824267782426</v>
       </c>
     </row>
     <row r="21">
@@ -37531,7 +37745,10 @@
         <v>0.133333333333326</v>
       </c>
       <c r="FE21">
-        <v>0</v>
+        <v>-0.133333333333326</v>
+      </c>
+      <c r="FF21">
+        <v>-0.199468085106372</v>
       </c>
     </row>
     <row r="22">
@@ -38020,6 +38237,9 @@
       <c r="FE22">
         <v>0.645161290322585</v>
       </c>
+      <c r="FF22">
+        <v>0.955180014695086</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -38507,6 +38727,9 @@
       <c r="FE23">
         <v>-0.180722891566272</v>
       </c>
+      <c r="FF23">
+        <v>-0.240673886883259</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -38994,6 +39217,9 @@
       <c r="FE24">
         <v>-0.0653167864141233</v>
       </c>
+      <c r="FF24">
+        <v>-0.0657894736842068</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -39479,7 +39705,10 @@
         <v>-0.80482897384307</v>
       </c>
       <c r="FE25">
-        <v>-1.60000000000001</v>
+        <v>-1.8</v>
+      </c>
+      <c r="FF25">
+        <v>-0.806451612903237</v>
       </c>
     </row>
     <row r="26">
@@ -39968,6 +40197,9 @@
       <c r="FE26">
         <v>0.566695727986043</v>
       </c>
+      <c r="FF26">
+        <v>0.435161009573542</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -40455,6 +40687,9 @@
       <c r="FE27">
         <v>0.359138068635266</v>
       </c>
+      <c r="FF27">
+        <v>0.319106501794979</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -40942,6 +41177,9 @@
       <c r="FE28">
         <v>2.90033940141931</v>
       </c>
+      <c r="FF28">
+        <v>2.63242375601926</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -41429,6 +41667,9 @@
       <c r="FE29">
         <v>0.869963369963373</v>
       </c>
+      <c r="FF29">
+        <v>1.5895278167368</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -41916,6 +42157,9 @@
       <c r="FE30">
         <v>0.38461538461539</v>
       </c>
+      <c r="FF30">
+        <v>2.07509881422926</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -42403,6 +42647,9 @@
       <c r="FE31" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FF31" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -42890,6 +43137,9 @@
       <c r="FE32">
         <v>-1.15473441108545</v>
       </c>
+      <c r="FF32">
+        <v>-1.1389521640091</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -43377,6 +43627,9 @@
       <c r="FE33">
         <v>1.23966942148761</v>
       </c>
+      <c r="FF33">
+        <v>0.10235414534291</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -43862,7 +44115,10 @@
         <v>0.447427293064867</v>
       </c>
       <c r="FE34">
-        <v>-0.335195530726254</v>
+        <v>-0.446927374301682</v>
+      </c>
+      <c r="FF34">
+        <v>-0.222965440356748</v>
       </c>
     </row>
     <row r="35">
@@ -44349,7 +44605,10 @@
         <v>-3.73626373626374</v>
       </c>
       <c r="FE35">
-        <v>-3.77777777777778</v>
+        <v>-2.44444444444445</v>
+      </c>
+      <c r="FF35">
+        <v>-2.53456221198157</v>
       </c>
     </row>
     <row r="36">
@@ -44836,7 +45095,10 @@
         <v>0.266429840142089</v>
       </c>
       <c r="FE36">
-        <v>0.472394449365193</v>
+        <v>0.442869796279877</v>
+      </c>
+      <c r="FF36">
+        <v>1.02317183268134</v>
       </c>
     </row>
     <row r="37">
@@ -45323,7 +45585,10 @@
         <v>-0.981595092024536</v>
       </c>
       <c r="FE37">
-        <v>-1.96560196560198</v>
+        <v>-0.368550368550382</v>
+      </c>
+      <c r="FF37">
+        <v>-0.7416563658838</v>
       </c>
     </row>
     <row r="38">
@@ -45810,7 +46075,10 @@
         <v>1.63720660678065</v>
       </c>
       <c r="FE38">
-        <v>0.880866425992767</v>
+        <v>0.967509025270748</v>
+      </c>
+      <c r="FF38">
+        <v>0.955137481910278</v>
       </c>
     </row>
     <row r="39">
@@ -46299,6 +46567,9 @@
       <c r="FE39">
         <v>0.0861573808156265</v>
       </c>
+      <c r="FF39">
+        <v>0.144175317185714</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -46786,6 +47057,9 @@
       <c r="FE40">
         <v>1.48883374689827</v>
       </c>
+      <c r="FF40">
+        <v>1.74563591022445</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -47271,7 +47545,10 @@
         <v>1.24019235636547</v>
       </c>
       <c r="FE41">
-        <v>-0.576441102756895</v>
+        <v>-0.601503759398491</v>
+      </c>
+      <c r="FF41">
+        <v>-1.55850792028614</v>
       </c>
     </row>
     <row r="42">
@@ -47760,6 +48037,9 @@
       <c r="FE42">
         <v>1.27388535031847</v>
       </c>
+      <c r="FF42">
+        <v>1.21250797702617</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -48247,6 +48527,9 @@
       <c r="FE43">
         <v>-2.32067510548524</v>
       </c>
+      <c r="FF43">
+        <v>-2.51748251748251</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -48734,6 +49017,9 @@
       <c r="FE44">
         <v>0.383367738130332</v>
       </c>
+      <c r="FF44">
+        <v>0.444312796208548</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -49221,6 +49507,9 @@
       <c r="FE45">
         <v>-0.662251655629137</v>
       </c>
+      <c r="FF45">
+        <v>-0.687285223367707</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -49706,7 +49995,10 @@
         <v>2.71206001154067</v>
       </c>
       <c r="FE46">
-        <v>2.13872832369942</v>
+        <v>2.19653179190752</v>
+      </c>
+      <c r="FF46">
+        <v>0.176991150442485</v>
       </c>
     </row>
     <row r="47">
@@ -50195,6 +50487,9 @@
       <c r="FE47">
         <v>-0.767263427109985</v>
       </c>
+      <c r="FF47">
+        <v>-1.03359173126616</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -50682,6 +50977,9 @@
       <c r="FE48">
         <v>2.15355805243447</v>
       </c>
+      <c r="FF48">
+        <v>2.0408163265306</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -51167,7 +51465,10 @@
         <v>0.674730519213367</v>
       </c>
       <c r="FE49">
-        <v>0.710098257782174</v>
+        <v>0.825695648583932</v>
+      </c>
+      <c r="FF49">
+        <v>0.835470262221847</v>
       </c>
     </row>
     <row r="50">
@@ -51656,6 +51957,9 @@
       <c r="FE50">
         <v>0.591278640059115</v>
       </c>
+      <c r="FF50">
+        <v>0.443786982248538</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -52141,7 +52445,10 @@
         <v>0.303030303030307</v>
       </c>
       <c r="FE51">
-        <v>-1.80722891566265</v>
+        <v>-1.50602409638554</v>
+      </c>
+      <c r="FF51">
+        <v>-3.53697749196142</v>
       </c>
     </row>
     <row r="52">
@@ -52628,7 +52935,10 @@
         <v>3.21167883211679</v>
       </c>
       <c r="FE52">
-        <v>2.76323443862713</v>
+        <v>2.76323443862711</v>
+      </c>
+      <c r="FF52">
+        <v>2.83836271287719</v>
       </c>
     </row>
     <row r="53">
@@ -53115,7 +53425,10 @@
         <v>-0.630563798219601</v>
       </c>
       <c r="FE53">
-        <v>-0.890207715133523</v>
+        <v>-0.927299703264095</v>
+      </c>
+      <c r="FF53">
+        <v>-0.957995578481933</v>
       </c>
     </row>
     <row r="54">
@@ -53604,6 +53917,9 @@
       <c r="FE54">
         <v>-1.57232704402515</v>
       </c>
+      <c r="FF54">
+        <v>-1.10584518167457</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -54089,7 +54405,10 @@
         <v>-1.86219739292364</v>
       </c>
       <c r="FE55">
-        <v>-2.22737819025523</v>
+        <v>-2.18097447795823</v>
+      </c>
+      <c r="FF55">
+        <v>1.01941747572815</v>
       </c>
     </row>
     <row r="56">
@@ -54576,7 +54895,10 @@
         <v>0.317460317460311</v>
       </c>
       <c r="FE56">
-        <v>0.319488817891367</v>
+        <v>0.638977635782745</v>
+      </c>
+      <c r="FF56">
+        <v>1.28205128205129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
SEM Update on July 21 2026
</commit_message>
<xml_diff>
--- a/static/data/source/state_and_local_public_education_employment.xlsx
+++ b/static/data/source/state_and_local_public_education_employment.xlsx
@@ -370,7 +370,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A4:FR56"/>
+  <dimension ref="A4:FS56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="4">
@@ -1244,6 +1244,11 @@
           <t>05/01/2026</t>
         </is>
       </c>
+      <c r="FS4" t="inlineStr">
+        <is>
+          <t>06/01/2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1765,10 +1770,13 @@
         <v>11275.1</v>
       </c>
       <c r="FQ5">
-        <v>11248.4</v>
+        <v>11247.2</v>
       </c>
       <c r="FR5">
-        <v>11095</v>
+        <v>11091.6</v>
+      </c>
+      <c r="FS5">
+        <v>10466.7</v>
       </c>
     </row>
     <row r="6">
@@ -2296,6 +2304,9 @@
       <c r="FR6">
         <v>186</v>
       </c>
+      <c r="FS6">
+        <v>182.7</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2820,7 +2831,10 @@
         <v>27.9</v>
       </c>
       <c r="FR7">
-        <v>27</v>
+        <v>26.8</v>
+      </c>
+      <c r="FS7">
+        <v>22.2</v>
       </c>
     </row>
     <row r="8">
@@ -3346,7 +3360,10 @@
         <v>200.6</v>
       </c>
       <c r="FR8">
-        <v>188</v>
+        <v>187.7</v>
+      </c>
+      <c r="FS8">
+        <v>149.4</v>
       </c>
     </row>
     <row r="9">
@@ -3874,6 +3891,9 @@
       <c r="FR9">
         <v>97.1</v>
       </c>
+      <c r="FS9">
+        <v>89.5</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4398,7 +4418,10 @@
         <v>1295</v>
       </c>
       <c r="FR10">
-        <v>1300.7</v>
+        <v>1298.4</v>
+      </c>
+      <c r="FS10">
+        <v>1265.6</v>
       </c>
     </row>
     <row r="11">
@@ -4924,7 +4947,10 @@
         <v>246.4</v>
       </c>
       <c r="FR11">
-        <v>246.3</v>
+        <v>245.9</v>
+      </c>
+      <c r="FS11">
+        <v>229.2</v>
       </c>
     </row>
     <row r="12">
@@ -5450,7 +5476,10 @@
         <v>125</v>
       </c>
       <c r="FR12">
-        <v>124.4</v>
+        <v>125.3</v>
+      </c>
+      <c r="FS12">
+        <v>117.3</v>
       </c>
     </row>
     <row r="13">
@@ -5976,7 +6005,10 @@
         <v>39.4</v>
       </c>
       <c r="FR13">
-        <v>38.7</v>
+        <v>39.5</v>
+      </c>
+      <c r="FS13">
+        <v>37.2</v>
       </c>
     </row>
     <row r="14">
@@ -6504,6 +6536,9 @@
       <c r="FR14" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FS14" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7030,6 +7065,9 @@
       <c r="FR15">
         <v>485.4</v>
       </c>
+      <c r="FS15">
+        <v>405.7</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -7554,7 +7592,10 @@
         <v>353.9</v>
       </c>
       <c r="FR16">
-        <v>351.5</v>
+        <v>351.2</v>
+      </c>
+      <c r="FS16">
+        <v>335.7</v>
       </c>
     </row>
     <row r="17">
@@ -8082,6 +8123,9 @@
       <c r="FR17" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FS17" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -8606,7 +8650,10 @@
         <v>64</v>
       </c>
       <c r="FR18">
-        <v>61.8</v>
+        <v>61.7</v>
+      </c>
+      <c r="FS18">
+        <v>58.1</v>
       </c>
     </row>
     <row r="19">
@@ -9132,7 +9179,10 @@
         <v>470.8</v>
       </c>
       <c r="FR19">
-        <v>467</v>
+        <v>466.9</v>
+      </c>
+      <c r="FS19">
+        <v>429</v>
       </c>
     </row>
     <row r="20">
@@ -9658,7 +9708,10 @@
         <v>227.3</v>
       </c>
       <c r="FR20">
-        <v>222.8</v>
+        <v>222.5</v>
+      </c>
+      <c r="FS20">
+        <v>182.2</v>
       </c>
     </row>
     <row r="21">
@@ -10184,7 +10237,10 @@
         <v>149.8</v>
       </c>
       <c r="FR21">
-        <v>150.1</v>
+        <v>149.2</v>
+      </c>
+      <c r="FS21">
+        <v>134.8</v>
       </c>
     </row>
     <row r="22">
@@ -10712,6 +10768,9 @@
       <c r="FR22">
         <v>137.4</v>
       </c>
+      <c r="FS22">
+        <v>122.2</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -11236,7 +11295,10 @@
         <v>165.7</v>
       </c>
       <c r="FR23">
-        <v>165.8</v>
+        <v>165.7</v>
+      </c>
+      <c r="FS23">
+        <v>155.1</v>
       </c>
     </row>
     <row r="24">
@@ -11764,6 +11826,9 @@
       <c r="FR24">
         <v>151.9</v>
       </c>
+      <c r="FS24">
+        <v>140.8</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -12290,6 +12355,9 @@
       <c r="FR25">
         <v>49.2</v>
       </c>
+      <c r="FS25">
+        <v>48</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -12816,6 +12884,9 @@
       <c r="FR26">
         <v>230.8</v>
       </c>
+      <c r="FS26">
+        <v>214.9</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -13342,6 +13413,9 @@
       <c r="FR27">
         <v>251.5</v>
       </c>
+      <c r="FS27">
+        <v>244.4</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -13868,6 +13942,9 @@
       <c r="FR28">
         <v>319.7</v>
       </c>
+      <c r="FS28">
+        <v>305</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -14394,6 +14471,9 @@
       <c r="FR29">
         <v>217.3</v>
       </c>
+      <c r="FS29">
+        <v>205.7</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -14918,7 +14998,10 @@
         <v>104.4</v>
       </c>
       <c r="FR30">
-        <v>103.3</v>
+        <v>103.4</v>
+      </c>
+      <c r="FS30">
+        <v>98.9</v>
       </c>
     </row>
     <row r="31">
@@ -15446,6 +15529,9 @@
       <c r="FR31" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FS31" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -15972,6 +16058,9 @@
       <c r="FR32">
         <v>43.4</v>
       </c>
+      <c r="FS32">
+        <v>41.3</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -16496,7 +16585,10 @@
         <v>98</v>
       </c>
       <c r="FR33">
-        <v>97.8</v>
+        <v>97.6</v>
+      </c>
+      <c r="FS33">
+        <v>90.7</v>
       </c>
     </row>
     <row r="34">
@@ -17022,7 +17114,10 @@
         <v>89.1</v>
       </c>
       <c r="FR34">
-        <v>89.5</v>
+        <v>89.9</v>
+      </c>
+      <c r="FS34">
+        <v>79.4</v>
       </c>
     </row>
     <row r="35">
@@ -17548,7 +17643,10 @@
         <v>43.9</v>
       </c>
       <c r="FR35">
-        <v>42.3</v>
+        <v>42.4</v>
+      </c>
+      <c r="FS35">
+        <v>38.3</v>
       </c>
     </row>
     <row r="36">
@@ -18074,7 +18172,10 @@
         <v>340.2</v>
       </c>
       <c r="FR36">
-        <v>335.7</v>
+        <v>335.3</v>
+      </c>
+      <c r="FS36">
+        <v>325.5</v>
       </c>
     </row>
     <row r="37">
@@ -18602,6 +18703,9 @@
       <c r="FR37">
         <v>80.3</v>
       </c>
+      <c r="FS37">
+        <v>72.4</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -19126,7 +19230,10 @@
         <v>699.2</v>
       </c>
       <c r="FR38">
-        <v>697.6</v>
+        <v>702.8</v>
+      </c>
+      <c r="FS38">
+        <v>695.9</v>
       </c>
     </row>
     <row r="39">
@@ -19654,6 +19761,9 @@
       <c r="FR39">
         <v>347.3</v>
       </c>
+      <c r="FS39">
+        <v>319.6</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -20180,6 +20290,9 @@
       <c r="FR40">
         <v>40.8</v>
       </c>
+      <c r="FS40">
+        <v>35.6</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -20704,7 +20817,10 @@
         <v>396.6</v>
       </c>
       <c r="FR41">
-        <v>385.3</v>
+        <v>385.1</v>
+      </c>
+      <c r="FS41">
+        <v>360.3</v>
       </c>
     </row>
     <row r="42">
@@ -21232,6 +21348,9 @@
       <c r="FR42">
         <v>158.6</v>
       </c>
+      <c r="FS42">
+        <v>145.6</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -21756,7 +21875,10 @@
         <v>138.9</v>
       </c>
       <c r="FR43">
-        <v>139.4</v>
+        <v>139.3</v>
+      </c>
+      <c r="FS43">
+        <v>136.5</v>
       </c>
     </row>
     <row r="44">
@@ -22282,7 +22404,10 @@
         <v>340.4</v>
       </c>
       <c r="FR44">
-        <v>339.1</v>
+        <v>339.6</v>
+      </c>
+      <c r="FS44">
+        <v>313.7</v>
       </c>
     </row>
     <row r="45">
@@ -22810,6 +22935,9 @@
       <c r="FR45">
         <v>28.9</v>
       </c>
+      <c r="FS45">
+        <v>26.9</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -23334,7 +23462,10 @@
         <v>176.8</v>
       </c>
       <c r="FR46">
-        <v>169.8</v>
+        <v>170.3</v>
+      </c>
+      <c r="FS46">
+        <v>167.8</v>
       </c>
     </row>
     <row r="47">
@@ -23862,6 +23993,9 @@
       <c r="FR47">
         <v>38.3</v>
       </c>
+      <c r="FS47">
+        <v>34.5</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -24388,6 +24522,9 @@
       <c r="FR48">
         <v>215</v>
       </c>
+      <c r="FS48">
+        <v>201</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -24912,7 +25049,10 @@
         <v>1221.1</v>
       </c>
       <c r="FR49">
-        <v>1219</v>
+        <v>1218</v>
+      </c>
+      <c r="FS49">
+        <v>1164.4</v>
       </c>
     </row>
     <row r="50">
@@ -25440,6 +25580,9 @@
       <c r="FR50">
         <v>135.8</v>
       </c>
+      <c r="FS50">
+        <v>128.3</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -25964,7 +26107,10 @@
         <v>32.7</v>
       </c>
       <c r="FR51">
-        <v>30</v>
+        <v>29.9</v>
+      </c>
+      <c r="FS51">
+        <v>29.6</v>
       </c>
     </row>
     <row r="52">
@@ -26490,7 +26636,10 @@
         <v>353.3</v>
       </c>
       <c r="FR52">
-        <v>344.2</v>
+        <v>344.3</v>
+      </c>
+      <c r="FS52">
+        <v>336</v>
       </c>
     </row>
     <row r="53">
@@ -27018,6 +27167,9 @@
       <c r="FR53">
         <v>268.8</v>
       </c>
+      <c r="FS53">
+        <v>262.9</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -27542,7 +27694,10 @@
         <v>62.6</v>
       </c>
       <c r="FR54">
-        <v>62.6</v>
+        <v>62.7</v>
+      </c>
+      <c r="FS54">
+        <v>56.9</v>
       </c>
     </row>
     <row r="55">
@@ -28070,6 +28225,9 @@
       <c r="FR55">
         <v>208.1</v>
       </c>
+      <c r="FS55">
+        <v>186.7</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -28594,7 +28752,10 @@
         <v>31.5</v>
       </c>
       <c r="FR56">
-        <v>31.6</v>
+        <v>31.4</v>
+      </c>
+      <c r="FS56">
+        <v>28.9</v>
       </c>
     </row>
   </sheetData>
@@ -28606,7 +28767,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A4:FF56"/>
+  <dimension ref="A4:FG56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="4">
@@ -29420,6 +29581,11 @@
           <t>05/01/2026</t>
         </is>
       </c>
+      <c r="FG4" t="inlineStr">
+        <is>
+          <t>06/01/2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -29905,10 +30071,13 @@
         <v>-0.083300101909712</v>
       </c>
       <c r="FE5">
-        <v>-0.261573519892888</v>
+        <v>-0.272213798668182</v>
       </c>
       <c r="FF5">
-        <v>-0.0603511173964413</v>
+        <v>-0.0909770575677632</v>
+      </c>
+      <c r="FG5">
+        <v>-0.356051446577999</v>
       </c>
     </row>
     <row r="6">
@@ -30400,6 +30569,9 @@
       <c r="FF6">
         <v>3.10421286031043</v>
       </c>
+      <c r="FG6">
+        <v>3.33710407239818</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -30888,7 +31060,10 @@
         <v>-2.78745644599303</v>
       </c>
       <c r="FF7">
-        <v>-2.87769784172662</v>
+        <v>-3.59712230215827</v>
+      </c>
+      <c r="FG7">
+        <v>-2.63157894736841</v>
       </c>
     </row>
     <row r="8">
@@ -31378,7 +31553,10 @@
         <v>-2.52672497570455</v>
       </c>
       <c r="FF8">
-        <v>-0.3709591944886</v>
+        <v>-0.529941706412295</v>
+      </c>
+      <c r="FG8">
+        <v>-1.45118733509234</v>
       </c>
     </row>
     <row r="9">
@@ -31870,6 +32048,9 @@
       <c r="FF9">
         <v>-0.614124872057313</v>
       </c>
+      <c r="FG9">
+        <v>-0.444938820912131</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -32358,7 +32539,10 @@
         <v>-2.07199032062917</v>
       </c>
       <c r="FF10">
-        <v>-1.75981873111784</v>
+        <v>-1.93353474320241</v>
+      </c>
+      <c r="FG10">
+        <v>-2.14180777855098</v>
       </c>
     </row>
     <row r="11">
@@ -32848,7 +33032,10 @@
         <v>1.73410404624277</v>
       </c>
       <c r="FF11">
-        <v>1.60891089108912</v>
+        <v>1.44389438943894</v>
+      </c>
+      <c r="FG11">
+        <v>2.45864997764865</v>
       </c>
     </row>
     <row r="12">
@@ -33338,7 +33525,10 @@
         <v>-1.41955835962145</v>
       </c>
       <c r="FF12">
-        <v>-1.34813639968279</v>
+        <v>-0.634417129262488</v>
+      </c>
+      <c r="FG12">
+        <v>-0.929054054054061</v>
       </c>
     </row>
     <row r="13">
@@ -33828,7 +34018,10 @@
         <v>-2.47524752475248</v>
       </c>
       <c r="FF13">
-        <v>-2.27272727272727</v>
+        <v>-0.252525252525256</v>
+      </c>
+      <c r="FG13">
+        <v>0.269541778975764</v>
       </c>
     </row>
     <row r="14">
@@ -34320,6 +34513,9 @@
       <c r="FF14" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FG14" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -34810,6 +35006,9 @@
       <c r="FF15">
         <v>-1.66126418152351</v>
       </c>
+      <c r="FG15">
+        <v>-1.43343051506318</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -35298,7 +35497,10 @@
         <v>0.511218403862542</v>
       </c>
       <c r="FF16">
-        <v>0.543478260869559</v>
+        <v>0.45766590389015</v>
+      </c>
+      <c r="FG16">
+        <v>0.328750747160796</v>
       </c>
     </row>
     <row r="17">
@@ -35790,6 +35992,9 @@
       <c r="FF17" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FG17" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -36278,7 +36483,10 @@
         <v>-0.311526479750783</v>
       </c>
       <c r="FF18">
-        <v>-1.12</v>
+        <v>-1.28</v>
+      </c>
+      <c r="FG18">
+        <v>-2.68006700167506</v>
       </c>
     </row>
     <row r="19">
@@ -36768,7 +36976,10 @@
         <v>0.965043963113875</v>
       </c>
       <c r="FF19">
-        <v>0.689952565761101</v>
+        <v>0.668391548081074</v>
+      </c>
+      <c r="FG19">
+        <v>-0.186133085155876</v>
       </c>
     </row>
     <row r="20">
@@ -37258,7 +37469,10 @@
         <v>-5.99669148056245</v>
       </c>
       <c r="FF20">
-        <v>-6.77824267782426</v>
+        <v>-6.90376569037657</v>
+      </c>
+      <c r="FG20">
+        <v>-8.67167919799499</v>
       </c>
     </row>
     <row r="21">
@@ -37748,7 +37962,10 @@
         <v>-0.133333333333326</v>
       </c>
       <c r="FF21">
-        <v>-0.199468085106372</v>
+        <v>-0.797872340425524</v>
+      </c>
+      <c r="FG21">
+        <v>-1.38990490124358</v>
       </c>
     </row>
     <row r="22">
@@ -38240,6 +38457,9 @@
       <c r="FF22">
         <v>0.955180014695086</v>
       </c>
+      <c r="FG22">
+        <v>0.493421052631574</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -38728,7 +38948,10 @@
         <v>-0.180722891566272</v>
       </c>
       <c r="FF23">
-        <v>-0.240673886883259</v>
+        <v>-0.300842358604091</v>
+      </c>
+      <c r="FG23">
+        <v>-0.385356454720613</v>
       </c>
     </row>
     <row r="24">
@@ -39220,6 +39443,9 @@
       <c r="FF24">
         <v>-0.0657894736842068</v>
       </c>
+      <c r="FG24">
+        <v>-0.070972320794886</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -39710,6 +39936,9 @@
       <c r="FF25">
         <v>-0.806451612903237</v>
       </c>
+      <c r="FG25">
+        <v>-1.23456790123457</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -40200,6 +40429,9 @@
       <c r="FF26">
         <v>0.435161009573542</v>
       </c>
+      <c r="FG26">
+        <v>0.844673862036595</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -40690,6 +40922,9 @@
       <c r="FF27">
         <v>0.319106501794979</v>
       </c>
+      <c r="FG27">
+        <v>0.287238407878546</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -41180,6 +41415,9 @@
       <c r="FF28">
         <v>2.63242375601926</v>
       </c>
+      <c r="FG28">
+        <v>2.93621329733378</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -41670,6 +41908,9 @@
       <c r="FF29">
         <v>1.5895278167368</v>
       </c>
+      <c r="FG29">
+        <v>0.882785679254542</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -42158,7 +42399,10 @@
         <v>0.38461538461539</v>
       </c>
       <c r="FF30">
-        <v>2.07509881422926</v>
+        <v>2.17391304347826</v>
+      </c>
+      <c r="FG30">
+        <v>1.43589743589744</v>
       </c>
     </row>
     <row r="31">
@@ -42650,6 +42894,9 @@
       <c r="FF31" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FG31" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -43140,6 +43387,9 @@
       <c r="FF32">
         <v>-1.1389521640091</v>
       </c>
+      <c r="FG32">
+        <v>-1.43198090692124</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -43628,7 +43878,10 @@
         <v>1.23966942148761</v>
       </c>
       <c r="FF33">
-        <v>0.10235414534291</v>
+        <v>-0.102354145342881</v>
+      </c>
+      <c r="FG33">
+        <v>0.0000000000000156679765327475</v>
       </c>
     </row>
     <row r="34">
@@ -44118,7 +44371,10 @@
         <v>-0.446927374301682</v>
       </c>
       <c r="FF34">
-        <v>-0.222965440356748</v>
+        <v>0.222965440356748</v>
+      </c>
+      <c r="FG34">
+        <v>5.4448871181939</v>
       </c>
     </row>
     <row r="35">
@@ -44608,7 +44864,10 @@
         <v>-2.44444444444445</v>
       </c>
       <c r="FF35">
-        <v>-2.53456221198157</v>
+        <v>-2.3041474654378</v>
+      </c>
+      <c r="FG35">
+        <v>-2.79187817258884</v>
       </c>
     </row>
     <row r="36">
@@ -45098,7 +45357,10 @@
         <v>0.442869796279877</v>
       </c>
       <c r="FF36">
-        <v>1.02317183268134</v>
+        <v>0.902798675895293</v>
+      </c>
+      <c r="FG36">
+        <v>0.68048252397154</v>
       </c>
     </row>
     <row r="37">
@@ -45590,6 +45852,9 @@
       <c r="FF37">
         <v>-0.7416563658838</v>
       </c>
+      <c r="FG37">
+        <v>0.83565459610029</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -46078,7 +46343,10 @@
         <v>0.967509025270748</v>
       </c>
       <c r="FF38">
-        <v>0.955137481910278</v>
+        <v>1.70767004341533</v>
+      </c>
+      <c r="FG38">
+        <v>1.72489402134192</v>
       </c>
     </row>
     <row r="39">
@@ -46570,6 +46838,9 @@
       <c r="FF39">
         <v>0.144175317185714</v>
       </c>
+      <c r="FG39">
+        <v>0.093955527716902</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -47060,6 +47331,9 @@
       <c r="FF40">
         <v>1.74563591022445</v>
       </c>
+      <c r="FG40">
+        <v>1.42450142450144</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -47548,7 +47822,10 @@
         <v>-0.601503759398491</v>
       </c>
       <c r="FF41">
-        <v>-1.55850792028614</v>
+        <v>-1.60960654062339</v>
+      </c>
+      <c r="FG41">
+        <v>0.0555401277422749</v>
       </c>
     </row>
     <row r="42">
@@ -48040,6 +48317,9 @@
       <c r="FF42">
         <v>1.21250797702617</v>
       </c>
+      <c r="FG42">
+        <v>1.32219902574809</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -48528,7 +48808,10 @@
         <v>-2.32067510548524</v>
       </c>
       <c r="FF43">
-        <v>-2.51748251748251</v>
+        <v>-2.58741258741258</v>
+      </c>
+      <c r="FG43">
+        <v>-2.84697508896797</v>
       </c>
     </row>
     <row r="44">
@@ -49018,7 +49301,10 @@
         <v>0.383367738130332</v>
       </c>
       <c r="FF44">
-        <v>0.444312796208548</v>
+        <v>0.592417061611391</v>
+      </c>
+      <c r="FG44">
+        <v>1.2588766946417</v>
       </c>
     </row>
     <row r="45">
@@ -49510,6 +49796,9 @@
       <c r="FF45">
         <v>-0.687285223367707</v>
       </c>
+      <c r="FG45">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -49998,7 +50287,10 @@
         <v>2.19653179190752</v>
       </c>
       <c r="FF46">
-        <v>0.176991150442485</v>
+        <v>0.471976401179948</v>
+      </c>
+      <c r="FG46">
+        <v>0.901984365604329</v>
       </c>
     </row>
     <row r="47">
@@ -50490,6 +50782,9 @@
       <c r="FF47">
         <v>-1.03359173126616</v>
       </c>
+      <c r="FG47">
+        <v>-0.5763688760807</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -50980,6 +51275,9 @@
       <c r="FF48">
         <v>2.0408163265306</v>
       </c>
+      <c r="FG48">
+        <v>1.41271442986883</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -51468,7 +51766,10 @@
         <v>0.825695648583932</v>
       </c>
       <c r="FF49">
-        <v>0.835470262221847</v>
+        <v>0.752750434279089</v>
+      </c>
+      <c r="FG49">
+        <v>0.232418008091594</v>
       </c>
     </row>
     <row r="50">
@@ -51960,6 +52261,9 @@
       <c r="FF50">
         <v>0.443786982248538</v>
       </c>
+      <c r="FG50">
+        <v>0.391236306729276</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -52448,7 +52752,10 @@
         <v>-1.50602409638554</v>
       </c>
       <c r="FF51">
-        <v>-3.53697749196142</v>
+        <v>-3.85852090032154</v>
+      </c>
+      <c r="FG51">
+        <v>0.0000000000000120024110770287</v>
       </c>
     </row>
     <row r="52">
@@ -52938,7 +53245,10 @@
         <v>2.76323443862711</v>
       </c>
       <c r="FF52">
-        <v>2.83836271287719</v>
+        <v>2.86824021511801</v>
+      </c>
+      <c r="FG52">
+        <v>2.56410256410256</v>
       </c>
     </row>
     <row r="53">
@@ -53430,6 +53740,9 @@
       <c r="FF53">
         <v>-0.957995578481933</v>
       </c>
+      <c r="FG53">
+        <v>-1.53558052434458</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -53918,7 +54231,10 @@
         <v>-1.57232704402515</v>
       </c>
       <c r="FF54">
-        <v>-1.10584518167457</v>
+        <v>-0.94786729857819</v>
+      </c>
+      <c r="FG54">
+        <v>-0.350262697022772</v>
       </c>
     </row>
     <row r="55">
@@ -54410,6 +54726,9 @@
       <c r="FF55">
         <v>1.01941747572815</v>
       </c>
+      <c r="FG55">
+        <v>-1.68509741969457</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -54898,7 +55217,10 @@
         <v>0.638977635782745</v>
       </c>
       <c r="FF56">
-        <v>1.28205128205129</v>
+        <v>0.641025641025639</v>
+      </c>
+      <c r="FG56">
+        <v>0.347222222222215</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
SEM Update on August 21
</commit_message>
<xml_diff>
--- a/static/data/source/state_and_local_public_education_employment.xlsx
+++ b/static/data/source/state_and_local_public_education_employment.xlsx
@@ -370,7 +370,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A4:FS56"/>
+  <dimension ref="A4:FT56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="4">
@@ -1249,6 +1249,11 @@
           <t>06/01/2026</t>
         </is>
       </c>
+      <c r="FT4" t="inlineStr">
+        <is>
+          <t>07/01/2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1773,10 +1778,13 @@
         <v>11247.2</v>
       </c>
       <c r="FR5">
-        <v>11091.6</v>
+        <v>11100.7</v>
       </c>
       <c r="FS5">
-        <v>10466.7</v>
+        <v>10454.8</v>
+      </c>
+      <c r="FT5">
+        <v>9328.6</v>
       </c>
     </row>
     <row r="6">
@@ -2305,7 +2313,10 @@
         <v>186</v>
       </c>
       <c r="FS6">
-        <v>182.7</v>
+        <v>182.6</v>
+      </c>
+      <c r="FT6">
+        <v>172</v>
       </c>
     </row>
     <row r="7">
@@ -2834,7 +2845,10 @@
         <v>26.8</v>
       </c>
       <c r="FS7">
-        <v>22.2</v>
+        <v>22.1</v>
+      </c>
+      <c r="FT7">
+        <v>18.5</v>
       </c>
     </row>
     <row r="8">
@@ -3363,7 +3377,10 @@
         <v>187.7</v>
       </c>
       <c r="FS8">
-        <v>149.4</v>
+        <v>150.1</v>
+      </c>
+      <c r="FT8">
+        <v>147.6</v>
       </c>
     </row>
     <row r="9">
@@ -3894,6 +3911,9 @@
       <c r="FS9">
         <v>89.5</v>
       </c>
+      <c r="FT9">
+        <v>78.4</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4423,6 +4443,9 @@
       <c r="FS10">
         <v>1265.6</v>
       </c>
+      <c r="FT10">
+        <v>1102.4</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4950,7 +4973,10 @@
         <v>245.9</v>
       </c>
       <c r="FS11">
-        <v>229.2</v>
+        <v>229.4</v>
+      </c>
+      <c r="FT11">
+        <v>215.3</v>
       </c>
     </row>
     <row r="12">
@@ -5481,6 +5507,9 @@
       <c r="FS12">
         <v>117.3</v>
       </c>
+      <c r="FT12">
+        <v>98</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6008,7 +6037,10 @@
         <v>39.5</v>
       </c>
       <c r="FS13">
-        <v>37.2</v>
+        <v>36.3</v>
+      </c>
+      <c r="FT13">
+        <v>34.5</v>
       </c>
     </row>
     <row r="14">
@@ -6539,6 +6571,9 @@
       <c r="FS14" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FT14" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7066,7 +7101,10 @@
         <v>485.4</v>
       </c>
       <c r="FS15">
-        <v>405.7</v>
+        <v>403.9</v>
+      </c>
+      <c r="FT15">
+        <v>396</v>
       </c>
     </row>
     <row r="16">
@@ -7595,7 +7633,10 @@
         <v>351.2</v>
       </c>
       <c r="FS16">
-        <v>335.7</v>
+        <v>336.2</v>
+      </c>
+      <c r="FT16">
+        <v>322</v>
       </c>
     </row>
     <row r="17">
@@ -8126,6 +8167,9 @@
       <c r="FS17" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FT17" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -8653,7 +8697,10 @@
         <v>61.7</v>
       </c>
       <c r="FS18">
-        <v>58.1</v>
+        <v>58.3</v>
+      </c>
+      <c r="FT18">
+        <v>52.9</v>
       </c>
     </row>
     <row r="19">
@@ -9182,7 +9229,10 @@
         <v>466.9</v>
       </c>
       <c r="FS19">
-        <v>429</v>
+        <v>429.2</v>
+      </c>
+      <c r="FT19">
+        <v>399.8</v>
       </c>
     </row>
     <row r="20">
@@ -9711,7 +9761,10 @@
         <v>222.5</v>
       </c>
       <c r="FS20">
-        <v>182.2</v>
+        <v>180.9</v>
+      </c>
+      <c r="FT20">
+        <v>165.4</v>
       </c>
     </row>
     <row r="21">
@@ -10240,7 +10293,10 @@
         <v>149.2</v>
       </c>
       <c r="FS21">
-        <v>134.8</v>
+        <v>136.5</v>
+      </c>
+      <c r="FT21">
+        <v>115.9</v>
       </c>
     </row>
     <row r="22">
@@ -10771,6 +10827,9 @@
       <c r="FS22">
         <v>122.2</v>
       </c>
+      <c r="FT22">
+        <v>99.9</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -11300,6 +11359,9 @@
       <c r="FS23">
         <v>155.1</v>
       </c>
+      <c r="FT23">
+        <v>129.9</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -11829,6 +11891,9 @@
       <c r="FS24">
         <v>140.8</v>
       </c>
+      <c r="FT24">
+        <v>133.3</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -12356,7 +12421,10 @@
         <v>49.2</v>
       </c>
       <c r="FS25">
-        <v>48</v>
+        <v>47.1</v>
+      </c>
+      <c r="FT25">
+        <v>40.2</v>
       </c>
     </row>
     <row r="26">
@@ -12887,6 +12955,9 @@
       <c r="FS26">
         <v>214.9</v>
       </c>
+      <c r="FT26">
+        <v>201.2</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -13416,6 +13487,9 @@
       <c r="FS27">
         <v>244.4</v>
       </c>
+      <c r="FT27">
+        <v>217.7</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -13945,6 +14019,9 @@
       <c r="FS28">
         <v>305</v>
       </c>
+      <c r="FT28">
+        <v>275.7</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -14472,7 +14549,10 @@
         <v>217.3</v>
       </c>
       <c r="FS29">
-        <v>205.7</v>
+        <v>205.5</v>
+      </c>
+      <c r="FT29">
+        <v>173.5</v>
       </c>
     </row>
     <row r="30">
@@ -15001,7 +15081,10 @@
         <v>103.4</v>
       </c>
       <c r="FS30">
-        <v>98.9</v>
+        <v>98.8</v>
+      </c>
+      <c r="FT30">
+        <v>93.1</v>
       </c>
     </row>
     <row r="31">
@@ -15532,6 +15615,9 @@
       <c r="FS31" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FT31" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -16061,6 +16147,9 @@
       <c r="FS32">
         <v>41.3</v>
       </c>
+      <c r="FT32">
+        <v>34.8</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -16588,7 +16677,10 @@
         <v>97.6</v>
       </c>
       <c r="FS33">
-        <v>90.7</v>
+        <v>90</v>
+      </c>
+      <c r="FT33">
+        <v>80.4</v>
       </c>
     </row>
     <row r="34">
@@ -17117,7 +17209,10 @@
         <v>89.9</v>
       </c>
       <c r="FS34">
-        <v>79.4</v>
+        <v>75.7</v>
+      </c>
+      <c r="FT34">
+        <v>72.5</v>
       </c>
     </row>
     <row r="35">
@@ -17646,7 +17741,10 @@
         <v>42.4</v>
       </c>
       <c r="FS35">
-        <v>38.3</v>
+        <v>39.8</v>
+      </c>
+      <c r="FT35">
+        <v>32.5</v>
       </c>
     </row>
     <row r="36">
@@ -18175,7 +18273,10 @@
         <v>335.3</v>
       </c>
       <c r="FS36">
-        <v>325.5</v>
+        <v>325.3</v>
+      </c>
+      <c r="FT36">
+        <v>266.7</v>
       </c>
     </row>
     <row r="37">
@@ -18704,7 +18805,10 @@
         <v>80.3</v>
       </c>
       <c r="FS37">
-        <v>72.4</v>
+        <v>70.9</v>
+      </c>
+      <c r="FT37">
+        <v>62.8</v>
       </c>
     </row>
     <row r="38">
@@ -19235,6 +19339,9 @@
       <c r="FS38">
         <v>695.9</v>
       </c>
+      <c r="FT38">
+        <v>580</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -19764,6 +19871,9 @@
       <c r="FS39">
         <v>319.6</v>
       </c>
+      <c r="FT39">
+        <v>262.7</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -20291,7 +20401,10 @@
         <v>40.8</v>
       </c>
       <c r="FS40">
-        <v>35.6</v>
+        <v>35.3</v>
+      </c>
+      <c r="FT40">
+        <v>29.5</v>
       </c>
     </row>
     <row r="41">
@@ -20820,7 +20933,10 @@
         <v>385.1</v>
       </c>
       <c r="FS41">
-        <v>360.3</v>
+        <v>361.2</v>
+      </c>
+      <c r="FT41">
+        <v>347.1</v>
       </c>
     </row>
     <row r="42">
@@ -21351,6 +21467,9 @@
       <c r="FS42">
         <v>145.6</v>
       </c>
+      <c r="FT42">
+        <v>132.6</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -21878,7 +21997,10 @@
         <v>139.3</v>
       </c>
       <c r="FS43">
-        <v>136.5</v>
+        <v>136.3</v>
+      </c>
+      <c r="FT43">
+        <v>105.7</v>
       </c>
     </row>
     <row r="44">
@@ -22409,6 +22531,9 @@
       <c r="FS44">
         <v>313.7</v>
       </c>
+      <c r="FT44">
+        <v>279</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -22938,6 +23063,9 @@
       <c r="FS45">
         <v>26.9</v>
       </c>
+      <c r="FT45">
+        <v>22.9</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -23465,7 +23593,10 @@
         <v>170.3</v>
       </c>
       <c r="FS46">
-        <v>167.8</v>
+        <v>167.7</v>
+      </c>
+      <c r="FT46">
+        <v>160.3</v>
       </c>
     </row>
     <row r="47">
@@ -23994,7 +24125,10 @@
         <v>38.3</v>
       </c>
       <c r="FS47">
-        <v>34.5</v>
+        <v>34</v>
+      </c>
+      <c r="FT47">
+        <v>28.2</v>
       </c>
     </row>
     <row r="48">
@@ -24523,7 +24657,10 @@
         <v>215</v>
       </c>
       <c r="FS48">
-        <v>201</v>
+        <v>202.1</v>
+      </c>
+      <c r="FT48">
+        <v>178.2</v>
       </c>
     </row>
     <row r="49">
@@ -25052,7 +25189,10 @@
         <v>1218</v>
       </c>
       <c r="FS49">
-        <v>1164.4</v>
+        <v>1162.2</v>
+      </c>
+      <c r="FT49">
+        <v>1081.8</v>
       </c>
     </row>
     <row r="50">
@@ -25583,6 +25723,9 @@
       <c r="FS50">
         <v>128.3</v>
       </c>
+      <c r="FT50">
+        <v>111</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -26110,7 +26253,10 @@
         <v>29.9</v>
       </c>
       <c r="FS51">
-        <v>29.6</v>
+        <v>29.2</v>
+      </c>
+      <c r="FT51">
+        <v>25.5</v>
       </c>
     </row>
     <row r="52">
@@ -26639,7 +26785,10 @@
         <v>344.3</v>
       </c>
       <c r="FS52">
-        <v>336</v>
+        <v>337</v>
+      </c>
+      <c r="FT52">
+        <v>298.8</v>
       </c>
     </row>
     <row r="53">
@@ -27168,7 +27317,10 @@
         <v>268.8</v>
       </c>
       <c r="FS53">
-        <v>262.9</v>
+        <v>257.9</v>
+      </c>
+      <c r="FT53">
+        <v>236.8</v>
       </c>
     </row>
     <row r="54">
@@ -27697,7 +27849,10 @@
         <v>62.7</v>
       </c>
       <c r="FS54">
-        <v>56.9</v>
+        <v>58.6</v>
+      </c>
+      <c r="FT54">
+        <v>54</v>
       </c>
     </row>
     <row r="55">
@@ -28226,7 +28381,10 @@
         <v>208.1</v>
       </c>
       <c r="FS55">
-        <v>186.7</v>
+        <v>184.9</v>
+      </c>
+      <c r="FT55">
+        <v>170.7</v>
       </c>
     </row>
     <row r="56">
@@ -28755,7 +28913,10 @@
         <v>31.4</v>
       </c>
       <c r="FS56">
-        <v>28.9</v>
+        <v>27.9</v>
+      </c>
+      <c r="FT56">
+        <v>24.5</v>
       </c>
     </row>
   </sheetData>
@@ -28767,7 +28928,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A4:FG56"/>
+  <dimension ref="A4:FH56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="4">
@@ -29586,6 +29747,11 @@
           <t>06/01/2026</t>
         </is>
       </c>
+      <c r="FH4" t="inlineStr">
+        <is>
+          <t>07/01/2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -30074,10 +30240,13 @@
         <v>-0.272213798668182</v>
       </c>
       <c r="FF5">
-        <v>-0.0909770575677632</v>
+        <v>-0.00900762946215444</v>
       </c>
       <c r="FG5">
-        <v>-0.356051446577999</v>
+        <v>-0.469340543216469</v>
+      </c>
+      <c r="FH5">
+        <v>-0.565995501881326</v>
       </c>
     </row>
     <row r="6">
@@ -30570,7 +30739,10 @@
         <v>3.10421286031043</v>
       </c>
       <c r="FG6">
-        <v>3.33710407239818</v>
+        <v>3.28054298642535</v>
+      </c>
+      <c r="FH6">
+        <v>2.9940119760479</v>
       </c>
     </row>
     <row r="7">
@@ -31063,7 +31235,10 @@
         <v>-3.59712230215827</v>
       </c>
       <c r="FG7">
-        <v>-2.63157894736841</v>
+        <v>-3.07017543859649</v>
+      </c>
+      <c r="FH7">
+        <v>-1.06951871657756</v>
       </c>
     </row>
     <row r="8">
@@ -31556,7 +31731,10 @@
         <v>-0.529941706412295</v>
       </c>
       <c r="FG8">
-        <v>-1.45118733509234</v>
+        <v>-0.989445910290238</v>
+      </c>
+      <c r="FH8">
+        <v>-0.873069173942232</v>
       </c>
     </row>
     <row r="9">
@@ -32051,6 +32229,9 @@
       <c r="FG9">
         <v>-0.444938820912131</v>
       </c>
+      <c r="FH9">
+        <v>-0.633713561470215</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -32544,6 +32725,9 @@
       <c r="FG10">
         <v>-2.14180777855098</v>
       </c>
+      <c r="FH10">
+        <v>-0.675736552842578</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -33035,7 +33219,10 @@
         <v>1.44389438943894</v>
       </c>
       <c r="FG11">
-        <v>2.45864997764865</v>
+        <v>2.54805543138132</v>
+      </c>
+      <c r="FH11">
+        <v>1.60453043888626</v>
       </c>
     </row>
     <row r="12">
@@ -33530,6 +33717,9 @@
       <c r="FG12">
         <v>-0.929054054054061</v>
       </c>
+      <c r="FH12">
+        <v>-0.709219858156017</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -34021,7 +34211,10 @@
         <v>-0.252525252525256</v>
       </c>
       <c r="FG13">
-        <v>0.269541778975764</v>
+        <v>-2.15633423180592</v>
+      </c>
+      <c r="FH13">
+        <v>-1.70940170940171</v>
       </c>
     </row>
     <row r="14">
@@ -34516,6 +34709,9 @@
       <c r="FG14" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FH14" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -35007,7 +35203,10 @@
         <v>-1.66126418152351</v>
       </c>
       <c r="FG15">
-        <v>-1.43343051506318</v>
+        <v>-1.87074829931974</v>
+      </c>
+      <c r="FH15">
+        <v>-1.36986301369863</v>
       </c>
     </row>
     <row r="16">
@@ -35500,7 +35699,10 @@
         <v>0.45766590389015</v>
       </c>
       <c r="FG16">
-        <v>0.328750747160796</v>
+        <v>0.478182904961154</v>
+      </c>
+      <c r="FH16">
+        <v>1.13065326633167</v>
       </c>
     </row>
     <row r="17">
@@ -35995,6 +36197,9 @@
       <c r="FG17" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FH17" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -36486,7 +36691,10 @@
         <v>-1.28</v>
       </c>
       <c r="FG18">
-        <v>-2.68006700167506</v>
+        <v>-2.34505862646566</v>
+      </c>
+      <c r="FH18">
+        <v>-1.85528756957328</v>
       </c>
     </row>
     <row r="19">
@@ -36979,7 +37187,10 @@
         <v>0.668391548081074</v>
       </c>
       <c r="FG19">
-        <v>-0.186133085155876</v>
+        <v>-0.139599813866894</v>
+      </c>
+      <c r="FH19">
+        <v>1.11279716742539</v>
       </c>
     </row>
     <row r="20">
@@ -37472,7 +37683,10 @@
         <v>-6.90376569037657</v>
       </c>
       <c r="FG20">
-        <v>-8.67167919799499</v>
+        <v>-9.32330827067669</v>
+      </c>
+      <c r="FH20">
+        <v>-5.48571428571428</v>
       </c>
     </row>
     <row r="21">
@@ -37965,7 +38179,10 @@
         <v>-0.797872340425524</v>
       </c>
       <c r="FG21">
-        <v>-1.38990490124358</v>
+        <v>-0.146305779078265</v>
+      </c>
+      <c r="FH21">
+        <v>1.0462074978204</v>
       </c>
     </row>
     <row r="22">
@@ -38460,6 +38677,9 @@
       <c r="FG22">
         <v>0.493421052631574</v>
       </c>
+      <c r="FH22">
+        <v>0.200601805416237</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -38953,6 +39173,9 @@
       <c r="FG23">
         <v>-0.385356454720613</v>
       </c>
+      <c r="FH23">
+        <v>-0.612088752869153</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -39446,6 +39669,9 @@
       <c r="FG24">
         <v>-0.070972320794886</v>
       </c>
+      <c r="FH24">
+        <v>-0.0749625187406041</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -39937,7 +40163,10 @@
         <v>-0.806451612903237</v>
       </c>
       <c r="FG25">
-        <v>-1.23456790123457</v>
+        <v>-3.08641975308642</v>
+      </c>
+      <c r="FH25">
+        <v>3.87596899224806</v>
       </c>
     </row>
     <row r="26">
@@ -40432,6 +40661,9 @@
       <c r="FG26">
         <v>0.844673862036595</v>
       </c>
+      <c r="FH26">
+        <v>1.00401606425701</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -40925,6 +41157,9 @@
       <c r="FG27">
         <v>0.287238407878546</v>
       </c>
+      <c r="FH27">
+        <v>0.184077312471227</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -41418,6 +41653,9 @@
       <c r="FG28">
         <v>2.93621329733378</v>
       </c>
+      <c r="FH28">
+        <v>3.25842696629215</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -41909,7 +42147,10 @@
         <v>1.5895278167368</v>
       </c>
       <c r="FG29">
-        <v>0.882785679254542</v>
+        <v>0.784698381559585</v>
+      </c>
+      <c r="FH29">
+        <v>1.46198830409357</v>
       </c>
     </row>
     <row r="30">
@@ -42402,7 +42643,10 @@
         <v>2.17391304347826</v>
       </c>
       <c r="FG30">
-        <v>1.43589743589744</v>
+        <v>1.33333333333335</v>
+      </c>
+      <c r="FH30">
+        <v>2.42024202420242</v>
       </c>
     </row>
     <row r="31">
@@ -42897,6 +43141,9 @@
       <c r="FG31" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FH31" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -43390,6 +43637,9 @@
       <c r="FG32">
         <v>-1.43198090692124</v>
       </c>
+      <c r="FH32">
+        <v>-1.41643059490085</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -43881,7 +44131,10 @@
         <v>-0.102354145342881</v>
       </c>
       <c r="FG33">
-        <v>0.0000000000000156679765327475</v>
+        <v>-0.771775082690175</v>
+      </c>
+      <c r="FH33">
+        <v>0.124533001245341</v>
       </c>
     </row>
     <row r="34">
@@ -44374,7 +44627,10 @@
         <v>0.222965440356748</v>
       </c>
       <c r="FG34">
-        <v>5.4448871181939</v>
+        <v>0.531208499335978</v>
+      </c>
+      <c r="FH34">
+        <v>0.554785020804446</v>
       </c>
     </row>
     <row r="35">
@@ -44867,7 +45123,10 @@
         <v>-2.3041474654378</v>
       </c>
       <c r="FG35">
-        <v>-2.79187817258884</v>
+        <v>1.01522842639595</v>
+      </c>
+      <c r="FH35">
+        <v>3.17460317460317</v>
       </c>
     </row>
     <row r="36">
@@ -45360,7 +45619,10 @@
         <v>0.902798675895293</v>
       </c>
       <c r="FG36">
-        <v>0.68048252397154</v>
+        <v>0.618620476337767</v>
+      </c>
+      <c r="FH36">
+        <v>0.489826676714398</v>
       </c>
     </row>
     <row r="37">
@@ -45853,7 +46115,10 @@
         <v>-0.7416563658838</v>
       </c>
       <c r="FG37">
-        <v>0.83565459610029</v>
+        <v>-1.25348189415041</v>
+      </c>
+      <c r="FH37">
+        <v>0.641025641025639</v>
       </c>
     </row>
     <row r="38">
@@ -46348,6 +46613,9 @@
       <c r="FG38">
         <v>1.72489402134192</v>
       </c>
+      <c r="FH38">
+        <v>2.43730130695866</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -46841,6 +47109,9 @@
       <c r="FG39">
         <v>0.093955527716902</v>
       </c>
+      <c r="FH39">
+        <v>0.0380807311500251</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -47332,7 +47603,10 @@
         <v>1.74563591022445</v>
       </c>
       <c r="FG40">
-        <v>1.42450142450144</v>
+        <v>0.569800569800578</v>
+      </c>
+      <c r="FH40">
+        <v>0.340136054421774</v>
       </c>
     </row>
     <row r="41">
@@ -47825,7 +48099,10 @@
         <v>-1.60960654062339</v>
       </c>
       <c r="FG41">
-        <v>0.0555401277422749</v>
+        <v>0.305470702582622</v>
+      </c>
+      <c r="FH41">
+        <v>-0.800228636753345</v>
       </c>
     </row>
     <row r="42">
@@ -48320,6 +48597,9 @@
       <c r="FG42">
         <v>1.32219902574809</v>
       </c>
+      <c r="FH42">
+        <v>1.45371078806427</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -48811,7 +49091,10 @@
         <v>-2.58741258741258</v>
       </c>
       <c r="FG43">
-        <v>-2.84697508896797</v>
+        <v>-2.98932384341636</v>
+      </c>
+      <c r="FH43">
+        <v>-2.93847566574838</v>
       </c>
     </row>
     <row r="44">
@@ -49306,6 +49589,9 @@
       <c r="FG44">
         <v>1.2588766946417</v>
       </c>
+      <c r="FH44">
+        <v>0.758396533044429</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -49799,6 +50085,9 @@
       <c r="FG45">
         <v>0</v>
       </c>
+      <c r="FH45">
+        <v>-1.7167381974249</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -50290,7 +50579,10 @@
         <v>0.471976401179948</v>
       </c>
       <c r="FG46">
-        <v>0.901984365604329</v>
+        <v>0.841852074564027</v>
+      </c>
+      <c r="FH46">
+        <v>1.84243964421857</v>
       </c>
     </row>
     <row r="47">
@@ -50783,7 +51075,10 @@
         <v>-1.03359173126616</v>
       </c>
       <c r="FG47">
-        <v>-0.5763688760807</v>
+        <v>-2.01729106628243</v>
+      </c>
+      <c r="FH47">
+        <v>-1.39860139860141</v>
       </c>
     </row>
     <row r="48">
@@ -51276,7 +51571,10 @@
         <v>2.0408163265306</v>
       </c>
       <c r="FG48">
-        <v>1.41271442986883</v>
+        <v>1.96770938446014</v>
+      </c>
+      <c r="FH48">
+        <v>2.23752151462994</v>
       </c>
     </row>
     <row r="49">
@@ -51769,7 +52067,10 @@
         <v>0.752750434279089</v>
       </c>
       <c r="FG49">
-        <v>0.232418008091594</v>
+        <v>0.0430403718688129</v>
+      </c>
+      <c r="FH49">
+        <v>-0.110803324099727</v>
       </c>
     </row>
     <row r="50">
@@ -52264,6 +52565,9 @@
       <c r="FG50">
         <v>0.391236306729276</v>
       </c>
+      <c r="FH50">
+        <v>-2.80210157618214</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -52755,7 +53059,10 @@
         <v>-3.85852090032154</v>
       </c>
       <c r="FG51">
-        <v>0.0000000000000120024110770287</v>
+        <v>-1.35135135135135</v>
+      </c>
+      <c r="FH51">
+        <v>6.25</v>
       </c>
     </row>
     <row r="52">
@@ -53248,7 +53555,10 @@
         <v>2.86824021511801</v>
       </c>
       <c r="FG52">
-        <v>2.56410256410256</v>
+        <v>2.86935286935286</v>
+      </c>
+      <c r="FH52">
+        <v>1.66723375297721</v>
       </c>
     </row>
     <row r="53">
@@ -53741,7 +54051,10 @@
         <v>-0.957995578481933</v>
       </c>
       <c r="FG53">
-        <v>-1.53558052434458</v>
+        <v>-3.40823970037454</v>
+      </c>
+      <c r="FH53">
+        <v>-2.99057763211798</v>
       </c>
     </row>
     <row r="54">
@@ -54234,7 +54547,10 @@
         <v>-0.94786729857819</v>
       </c>
       <c r="FG54">
-        <v>-0.350262697022772</v>
+        <v>2.62697022767074</v>
+      </c>
+      <c r="FH54">
+        <v>3.44827586206896</v>
       </c>
     </row>
     <row r="55">
@@ -54727,7 +55043,10 @@
         <v>1.01941747572815</v>
       </c>
       <c r="FG55">
-        <v>-1.68509741969457</v>
+        <v>-2.63296471827276</v>
+      </c>
+      <c r="FH55">
+        <v>-1.1008111239861</v>
       </c>
     </row>
     <row r="56">
@@ -55220,7 +55539,10 @@
         <v>0.641025641025639</v>
       </c>
       <c r="FG56">
-        <v>0.347222222222215</v>
+        <v>-3.12500000000001</v>
+      </c>
+      <c r="FH56">
+        <v>-3.92156862745098</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
SEM Fixed update on August 24
</commit_message>
<xml_diff>
--- a/static/data/source/state_and_local_public_education_employment.xlsx
+++ b/static/data/source/state_and_local_public_education_employment.xlsx
@@ -370,7 +370,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A4:FS56"/>
+  <dimension ref="A4:FT56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="4">
@@ -1249,6 +1249,11 @@
           <t>06/01/2026</t>
         </is>
       </c>
+      <c r="FT4" t="inlineStr">
+        <is>
+          <t>07/01/2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1773,10 +1778,13 @@
         <v>11247.2</v>
       </c>
       <c r="FR5">
-        <v>11091.6</v>
+        <v>11100.7</v>
       </c>
       <c r="FS5">
-        <v>10466.7</v>
+        <v>10454.8</v>
+      </c>
+      <c r="FT5">
+        <v>9328.6</v>
       </c>
     </row>
     <row r="6">
@@ -2305,7 +2313,10 @@
         <v>186</v>
       </c>
       <c r="FS6">
-        <v>182.7</v>
+        <v>182.6</v>
+      </c>
+      <c r="FT6">
+        <v>172</v>
       </c>
     </row>
     <row r="7">
@@ -2834,7 +2845,10 @@
         <v>26.8</v>
       </c>
       <c r="FS7">
-        <v>22.2</v>
+        <v>22.1</v>
+      </c>
+      <c r="FT7">
+        <v>18.5</v>
       </c>
     </row>
     <row r="8">
@@ -3363,7 +3377,10 @@
         <v>187.7</v>
       </c>
       <c r="FS8">
-        <v>149.4</v>
+        <v>150.1</v>
+      </c>
+      <c r="FT8">
+        <v>147.6</v>
       </c>
     </row>
     <row r="9">
@@ -3894,6 +3911,9 @@
       <c r="FS9">
         <v>89.5</v>
       </c>
+      <c r="FT9">
+        <v>78.4</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4423,6 +4443,9 @@
       <c r="FS10">
         <v>1265.6</v>
       </c>
+      <c r="FT10">
+        <v>1102.4</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4950,7 +4973,10 @@
         <v>245.9</v>
       </c>
       <c r="FS11">
-        <v>229.2</v>
+        <v>229.4</v>
+      </c>
+      <c r="FT11">
+        <v>215.3</v>
       </c>
     </row>
     <row r="12">
@@ -5481,6 +5507,9 @@
       <c r="FS12">
         <v>117.3</v>
       </c>
+      <c r="FT12">
+        <v>98</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6008,7 +6037,10 @@
         <v>39.5</v>
       </c>
       <c r="FS13">
-        <v>37.2</v>
+        <v>36.3</v>
+      </c>
+      <c r="FT13">
+        <v>34.5</v>
       </c>
     </row>
     <row r="14">
@@ -6539,6 +6571,9 @@
       <c r="FS14" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FT14" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7066,7 +7101,10 @@
         <v>485.4</v>
       </c>
       <c r="FS15">
-        <v>405.7</v>
+        <v>403.9</v>
+      </c>
+      <c r="FT15">
+        <v>396</v>
       </c>
     </row>
     <row r="16">
@@ -7595,7 +7633,10 @@
         <v>351.2</v>
       </c>
       <c r="FS16">
-        <v>335.7</v>
+        <v>336.2</v>
+      </c>
+      <c r="FT16">
+        <v>322</v>
       </c>
     </row>
     <row r="17">
@@ -8126,6 +8167,9 @@
       <c r="FS17" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FT17" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -8653,7 +8697,10 @@
         <v>61.7</v>
       </c>
       <c r="FS18">
-        <v>58.1</v>
+        <v>58.3</v>
+      </c>
+      <c r="FT18">
+        <v>52.9</v>
       </c>
     </row>
     <row r="19">
@@ -9182,7 +9229,10 @@
         <v>466.9</v>
       </c>
       <c r="FS19">
-        <v>429</v>
+        <v>429.2</v>
+      </c>
+      <c r="FT19">
+        <v>399.8</v>
       </c>
     </row>
     <row r="20">
@@ -9711,7 +9761,10 @@
         <v>222.5</v>
       </c>
       <c r="FS20">
-        <v>182.2</v>
+        <v>180.9</v>
+      </c>
+      <c r="FT20">
+        <v>165.4</v>
       </c>
     </row>
     <row r="21">
@@ -10240,7 +10293,10 @@
         <v>149.2</v>
       </c>
       <c r="FS21">
-        <v>134.8</v>
+        <v>136.5</v>
+      </c>
+      <c r="FT21">
+        <v>115.9</v>
       </c>
     </row>
     <row r="22">
@@ -10771,6 +10827,9 @@
       <c r="FS22">
         <v>122.2</v>
       </c>
+      <c r="FT22">
+        <v>99.9</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -11300,6 +11359,9 @@
       <c r="FS23">
         <v>155.1</v>
       </c>
+      <c r="FT23">
+        <v>129.9</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -11829,6 +11891,9 @@
       <c r="FS24">
         <v>140.8</v>
       </c>
+      <c r="FT24">
+        <v>133.3</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -12356,7 +12421,10 @@
         <v>49.2</v>
       </c>
       <c r="FS25">
-        <v>48</v>
+        <v>47.1</v>
+      </c>
+      <c r="FT25">
+        <v>40.2</v>
       </c>
     </row>
     <row r="26">
@@ -12887,6 +12955,9 @@
       <c r="FS26">
         <v>214.9</v>
       </c>
+      <c r="FT26">
+        <v>201.2</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -13416,6 +13487,9 @@
       <c r="FS27">
         <v>244.4</v>
       </c>
+      <c r="FT27">
+        <v>217.7</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -13945,6 +14019,9 @@
       <c r="FS28">
         <v>305</v>
       </c>
+      <c r="FT28">
+        <v>275.7</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -14472,7 +14549,10 @@
         <v>217.3</v>
       </c>
       <c r="FS29">
-        <v>205.7</v>
+        <v>205.5</v>
+      </c>
+      <c r="FT29">
+        <v>173.5</v>
       </c>
     </row>
     <row r="30">
@@ -15001,7 +15081,10 @@
         <v>103.4</v>
       </c>
       <c r="FS30">
-        <v>98.9</v>
+        <v>98.8</v>
+      </c>
+      <c r="FT30">
+        <v>93.1</v>
       </c>
     </row>
     <row r="31">
@@ -15532,6 +15615,9 @@
       <c r="FS31" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FT31" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -16061,6 +16147,9 @@
       <c r="FS32">
         <v>41.3</v>
       </c>
+      <c r="FT32">
+        <v>34.8</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -16588,7 +16677,10 @@
         <v>97.6</v>
       </c>
       <c r="FS33">
-        <v>90.7</v>
+        <v>90</v>
+      </c>
+      <c r="FT33">
+        <v>80.4</v>
       </c>
     </row>
     <row r="34">
@@ -17117,7 +17209,10 @@
         <v>89.9</v>
       </c>
       <c r="FS34">
-        <v>79.4</v>
+        <v>75.7</v>
+      </c>
+      <c r="FT34">
+        <v>72.5</v>
       </c>
     </row>
     <row r="35">
@@ -17646,7 +17741,10 @@
         <v>42.4</v>
       </c>
       <c r="FS35">
-        <v>38.3</v>
+        <v>39.8</v>
+      </c>
+      <c r="FT35">
+        <v>32.5</v>
       </c>
     </row>
     <row r="36">
@@ -18175,7 +18273,10 @@
         <v>335.3</v>
       </c>
       <c r="FS36">
-        <v>325.5</v>
+        <v>325.3</v>
+      </c>
+      <c r="FT36">
+        <v>266.7</v>
       </c>
     </row>
     <row r="37">
@@ -18704,7 +18805,10 @@
         <v>80.3</v>
       </c>
       <c r="FS37">
-        <v>72.4</v>
+        <v>70.9</v>
+      </c>
+      <c r="FT37">
+        <v>62.8</v>
       </c>
     </row>
     <row r="38">
@@ -19235,6 +19339,9 @@
       <c r="FS38">
         <v>695.9</v>
       </c>
+      <c r="FT38">
+        <v>580</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -19764,6 +19871,9 @@
       <c r="FS39">
         <v>319.6</v>
       </c>
+      <c r="FT39">
+        <v>262.7</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -20291,7 +20401,10 @@
         <v>40.8</v>
       </c>
       <c r="FS40">
-        <v>35.6</v>
+        <v>35.3</v>
+      </c>
+      <c r="FT40">
+        <v>29.5</v>
       </c>
     </row>
     <row r="41">
@@ -20820,7 +20933,10 @@
         <v>385.1</v>
       </c>
       <c r="FS41">
-        <v>360.3</v>
+        <v>361.2</v>
+      </c>
+      <c r="FT41">
+        <v>347.1</v>
       </c>
     </row>
     <row r="42">
@@ -21351,6 +21467,9 @@
       <c r="FS42">
         <v>145.6</v>
       </c>
+      <c r="FT42">
+        <v>132.6</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -21878,7 +21997,10 @@
         <v>139.3</v>
       </c>
       <c r="FS43">
-        <v>136.5</v>
+        <v>136.3</v>
+      </c>
+      <c r="FT43">
+        <v>105.7</v>
       </c>
     </row>
     <row r="44">
@@ -22409,6 +22531,9 @@
       <c r="FS44">
         <v>313.7</v>
       </c>
+      <c r="FT44">
+        <v>279</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -22938,6 +23063,9 @@
       <c r="FS45">
         <v>26.9</v>
       </c>
+      <c r="FT45">
+        <v>22.9</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -23465,7 +23593,10 @@
         <v>170.3</v>
       </c>
       <c r="FS46">
-        <v>167.8</v>
+        <v>167.7</v>
+      </c>
+      <c r="FT46">
+        <v>160.3</v>
       </c>
     </row>
     <row r="47">
@@ -23994,7 +24125,10 @@
         <v>38.3</v>
       </c>
       <c r="FS47">
-        <v>34.5</v>
+        <v>34</v>
+      </c>
+      <c r="FT47">
+        <v>28.2</v>
       </c>
     </row>
     <row r="48">
@@ -24523,7 +24657,10 @@
         <v>215</v>
       </c>
       <c r="FS48">
-        <v>201</v>
+        <v>202.1</v>
+      </c>
+      <c r="FT48">
+        <v>178.2</v>
       </c>
     </row>
     <row r="49">
@@ -25052,7 +25189,10 @@
         <v>1218</v>
       </c>
       <c r="FS49">
-        <v>1164.4</v>
+        <v>1162.2</v>
+      </c>
+      <c r="FT49">
+        <v>1081.8</v>
       </c>
     </row>
     <row r="50">
@@ -25583,6 +25723,9 @@
       <c r="FS50">
         <v>128.3</v>
       </c>
+      <c r="FT50">
+        <v>111</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -26110,7 +26253,10 @@
         <v>29.9</v>
       </c>
       <c r="FS51">
-        <v>29.6</v>
+        <v>29.2</v>
+      </c>
+      <c r="FT51">
+        <v>25.5</v>
       </c>
     </row>
     <row r="52">
@@ -26639,7 +26785,10 @@
         <v>344.3</v>
       </c>
       <c r="FS52">
-        <v>336</v>
+        <v>337</v>
+      </c>
+      <c r="FT52">
+        <v>298.8</v>
       </c>
     </row>
     <row r="53">
@@ -27168,7 +27317,10 @@
         <v>268.8</v>
       </c>
       <c r="FS53">
-        <v>262.9</v>
+        <v>257.9</v>
+      </c>
+      <c r="FT53">
+        <v>236.8</v>
       </c>
     </row>
     <row r="54">
@@ -27697,7 +27849,10 @@
         <v>62.7</v>
       </c>
       <c r="FS54">
-        <v>56.9</v>
+        <v>58.6</v>
+      </c>
+      <c r="FT54">
+        <v>54</v>
       </c>
     </row>
     <row r="55">
@@ -28226,7 +28381,10 @@
         <v>208.1</v>
       </c>
       <c r="FS55">
-        <v>186.7</v>
+        <v>184.9</v>
+      </c>
+      <c r="FT55">
+        <v>170.7</v>
       </c>
     </row>
     <row r="56">
@@ -28755,7 +28913,10 @@
         <v>31.4</v>
       </c>
       <c r="FS56">
-        <v>28.9</v>
+        <v>27.9</v>
+      </c>
+      <c r="FT56">
+        <v>24.5</v>
       </c>
     </row>
   </sheetData>
@@ -28767,7 +28928,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A4:FG56"/>
+  <dimension ref="A4:FH56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="4">
@@ -29586,6 +29747,11 @@
           <t>06/01/2026</t>
         </is>
       </c>
+      <c r="FH4" t="inlineStr">
+        <is>
+          <t>07/01/2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -30074,10 +30240,13 @@
         <v>-0.272213798668182</v>
       </c>
       <c r="FF5">
-        <v>-0.0909770575677632</v>
+        <v>-0.00900762946215444</v>
       </c>
       <c r="FG5">
-        <v>-0.356051446577999</v>
+        <v>-0.469340543216469</v>
+      </c>
+      <c r="FH5">
+        <v>-0.565995501881326</v>
       </c>
     </row>
     <row r="6">
@@ -30570,7 +30739,10 @@
         <v>3.10421286031043</v>
       </c>
       <c r="FG6">
-        <v>3.33710407239818</v>
+        <v>3.28054298642535</v>
+      </c>
+      <c r="FH6">
+        <v>2.9940119760479</v>
       </c>
     </row>
     <row r="7">
@@ -31063,7 +31235,10 @@
         <v>-3.59712230215827</v>
       </c>
       <c r="FG7">
-        <v>-2.63157894736841</v>
+        <v>-3.07017543859649</v>
+      </c>
+      <c r="FH7">
+        <v>-1.06951871657756</v>
       </c>
     </row>
     <row r="8">
@@ -31556,7 +31731,10 @@
         <v>-0.529941706412295</v>
       </c>
       <c r="FG8">
-        <v>-1.45118733509234</v>
+        <v>-0.989445910290238</v>
+      </c>
+      <c r="FH8">
+        <v>-0.873069173942232</v>
       </c>
     </row>
     <row r="9">
@@ -32051,6 +32229,9 @@
       <c r="FG9">
         <v>-0.444938820912131</v>
       </c>
+      <c r="FH9">
+        <v>-0.633713561470215</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -32544,6 +32725,9 @@
       <c r="FG10">
         <v>-2.14180777855098</v>
       </c>
+      <c r="FH10">
+        <v>-0.675736552842578</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -33035,7 +33219,10 @@
         <v>1.44389438943894</v>
       </c>
       <c r="FG11">
-        <v>2.45864997764865</v>
+        <v>2.54805543138132</v>
+      </c>
+      <c r="FH11">
+        <v>1.60453043888626</v>
       </c>
     </row>
     <row r="12">
@@ -33530,6 +33717,9 @@
       <c r="FG12">
         <v>-0.929054054054061</v>
       </c>
+      <c r="FH12">
+        <v>-0.709219858156017</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -34021,7 +34211,10 @@
         <v>-0.252525252525256</v>
       </c>
       <c r="FG13">
-        <v>0.269541778975764</v>
+        <v>-2.15633423180592</v>
+      </c>
+      <c r="FH13">
+        <v>-1.70940170940171</v>
       </c>
     </row>
     <row r="14">
@@ -34516,6 +34709,9 @@
       <c r="FG14" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FH14" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -35007,7 +35203,10 @@
         <v>-1.66126418152351</v>
       </c>
       <c r="FG15">
-        <v>-1.43343051506318</v>
+        <v>-1.87074829931974</v>
+      </c>
+      <c r="FH15">
+        <v>-1.36986301369863</v>
       </c>
     </row>
     <row r="16">
@@ -35500,7 +35699,10 @@
         <v>0.45766590389015</v>
       </c>
       <c r="FG16">
-        <v>0.328750747160796</v>
+        <v>0.478182904961154</v>
+      </c>
+      <c r="FH16">
+        <v>1.13065326633167</v>
       </c>
     </row>
     <row r="17">
@@ -35995,6 +36197,9 @@
       <c r="FG17" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FH17" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -36486,7 +36691,10 @@
         <v>-1.28</v>
       </c>
       <c r="FG18">
-        <v>-2.68006700167506</v>
+        <v>-2.34505862646566</v>
+      </c>
+      <c r="FH18">
+        <v>-1.85528756957328</v>
       </c>
     </row>
     <row r="19">
@@ -36979,7 +37187,10 @@
         <v>0.668391548081074</v>
       </c>
       <c r="FG19">
-        <v>-0.186133085155876</v>
+        <v>-0.139599813866894</v>
+      </c>
+      <c r="FH19">
+        <v>1.11279716742539</v>
       </c>
     </row>
     <row r="20">
@@ -37472,7 +37683,10 @@
         <v>-6.90376569037657</v>
       </c>
       <c r="FG20">
-        <v>-8.67167919799499</v>
+        <v>-9.32330827067669</v>
+      </c>
+      <c r="FH20">
+        <v>-5.48571428571428</v>
       </c>
     </row>
     <row r="21">
@@ -37965,7 +38179,10 @@
         <v>-0.797872340425524</v>
       </c>
       <c r="FG21">
-        <v>-1.38990490124358</v>
+        <v>-0.146305779078265</v>
+      </c>
+      <c r="FH21">
+        <v>1.0462074978204</v>
       </c>
     </row>
     <row r="22">
@@ -38460,6 +38677,9 @@
       <c r="FG22">
         <v>0.493421052631574</v>
       </c>
+      <c r="FH22">
+        <v>0.200601805416237</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -38953,6 +39173,9 @@
       <c r="FG23">
         <v>-0.385356454720613</v>
       </c>
+      <c r="FH23">
+        <v>-0.612088752869153</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -39446,6 +39669,9 @@
       <c r="FG24">
         <v>-0.070972320794886</v>
       </c>
+      <c r="FH24">
+        <v>-0.0749625187406041</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -39937,7 +40163,10 @@
         <v>-0.806451612903237</v>
       </c>
       <c r="FG25">
-        <v>-1.23456790123457</v>
+        <v>-3.08641975308642</v>
+      </c>
+      <c r="FH25">
+        <v>3.87596899224806</v>
       </c>
     </row>
     <row r="26">
@@ -40432,6 +40661,9 @@
       <c r="FG26">
         <v>0.844673862036595</v>
       </c>
+      <c r="FH26">
+        <v>1.00401606425701</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -40925,6 +41157,9 @@
       <c r="FG27">
         <v>0.287238407878546</v>
       </c>
+      <c r="FH27">
+        <v>0.184077312471227</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -41418,6 +41653,9 @@
       <c r="FG28">
         <v>2.93621329733378</v>
       </c>
+      <c r="FH28">
+        <v>3.25842696629215</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -41909,7 +42147,10 @@
         <v>1.5895278167368</v>
       </c>
       <c r="FG29">
-        <v>0.882785679254542</v>
+        <v>0.784698381559585</v>
+      </c>
+      <c r="FH29">
+        <v>1.46198830409357</v>
       </c>
     </row>
     <row r="30">
@@ -42402,7 +42643,10 @@
         <v>2.17391304347826</v>
       </c>
       <c r="FG30">
-        <v>1.43589743589744</v>
+        <v>1.33333333333335</v>
+      </c>
+      <c r="FH30">
+        <v>2.42024202420242</v>
       </c>
     </row>
     <row r="31">
@@ -42897,6 +43141,9 @@
       <c r="FG31" t="e">
         <v>#N/A</v>
       </c>
+      <c r="FH31" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -43390,6 +43637,9 @@
       <c r="FG32">
         <v>-1.43198090692124</v>
       </c>
+      <c r="FH32">
+        <v>-1.41643059490085</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -43881,7 +44131,10 @@
         <v>-0.102354145342881</v>
       </c>
       <c r="FG33">
-        <v>0.0000000000000156679765327475</v>
+        <v>-0.771775082690175</v>
+      </c>
+      <c r="FH33">
+        <v>0.124533001245341</v>
       </c>
     </row>
     <row r="34">
@@ -44374,7 +44627,10 @@
         <v>0.222965440356748</v>
       </c>
       <c r="FG34">
-        <v>5.4448871181939</v>
+        <v>0.531208499335978</v>
+      </c>
+      <c r="FH34">
+        <v>0.554785020804446</v>
       </c>
     </row>
     <row r="35">
@@ -44867,7 +45123,10 @@
         <v>-2.3041474654378</v>
       </c>
       <c r="FG35">
-        <v>-2.79187817258884</v>
+        <v>1.01522842639595</v>
+      </c>
+      <c r="FH35">
+        <v>3.17460317460317</v>
       </c>
     </row>
     <row r="36">
@@ -45360,7 +45619,10 @@
         <v>0.902798675895293</v>
       </c>
       <c r="FG36">
-        <v>0.68048252397154</v>
+        <v>0.618620476337767</v>
+      </c>
+      <c r="FH36">
+        <v>0.489826676714398</v>
       </c>
     </row>
     <row r="37">
@@ -45853,7 +46115,10 @@
         <v>-0.7416563658838</v>
       </c>
       <c r="FG37">
-        <v>0.83565459610029</v>
+        <v>-1.25348189415041</v>
+      </c>
+      <c r="FH37">
+        <v>0.641025641025639</v>
       </c>
     </row>
     <row r="38">
@@ -46348,6 +46613,9 @@
       <c r="FG38">
         <v>1.72489402134192</v>
       </c>
+      <c r="FH38">
+        <v>2.43730130695866</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -46841,6 +47109,9 @@
       <c r="FG39">
         <v>0.093955527716902</v>
       </c>
+      <c r="FH39">
+        <v>0.0380807311500251</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -47332,7 +47603,10 @@
         <v>1.74563591022445</v>
       </c>
       <c r="FG40">
-        <v>1.42450142450144</v>
+        <v>0.569800569800578</v>
+      </c>
+      <c r="FH40">
+        <v>0.340136054421774</v>
       </c>
     </row>
     <row r="41">
@@ -47825,7 +48099,10 @@
         <v>-1.60960654062339</v>
       </c>
       <c r="FG41">
-        <v>0.0555401277422749</v>
+        <v>0.305470702582622</v>
+      </c>
+      <c r="FH41">
+        <v>-0.800228636753345</v>
       </c>
     </row>
     <row r="42">
@@ -48320,6 +48597,9 @@
       <c r="FG42">
         <v>1.32219902574809</v>
       </c>
+      <c r="FH42">
+        <v>1.45371078806427</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -48811,7 +49091,10 @@
         <v>-2.58741258741258</v>
       </c>
       <c r="FG43">
-        <v>-2.84697508896797</v>
+        <v>-2.98932384341636</v>
+      </c>
+      <c r="FH43">
+        <v>-2.93847566574838</v>
       </c>
     </row>
     <row r="44">
@@ -49306,6 +49589,9 @@
       <c r="FG44">
         <v>1.2588766946417</v>
       </c>
+      <c r="FH44">
+        <v>0.758396533044429</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -49799,6 +50085,9 @@
       <c r="FG45">
         <v>0</v>
       </c>
+      <c r="FH45">
+        <v>-1.7167381974249</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -50290,7 +50579,10 @@
         <v>0.471976401179948</v>
       </c>
       <c r="FG46">
-        <v>0.901984365604329</v>
+        <v>0.841852074564027</v>
+      </c>
+      <c r="FH46">
+        <v>1.84243964421857</v>
       </c>
     </row>
     <row r="47">
@@ -50783,7 +51075,10 @@
         <v>-1.03359173126616</v>
       </c>
       <c r="FG47">
-        <v>-0.5763688760807</v>
+        <v>-2.01729106628243</v>
+      </c>
+      <c r="FH47">
+        <v>-1.39860139860141</v>
       </c>
     </row>
     <row r="48">
@@ -51276,7 +51571,10 @@
         <v>2.0408163265306</v>
       </c>
       <c r="FG48">
-        <v>1.41271442986883</v>
+        <v>1.96770938446014</v>
+      </c>
+      <c r="FH48">
+        <v>2.23752151462994</v>
       </c>
     </row>
     <row r="49">
@@ -51769,7 +52067,10 @@
         <v>0.752750434279089</v>
       </c>
       <c r="FG49">
-        <v>0.232418008091594</v>
+        <v>0.0430403718688129</v>
+      </c>
+      <c r="FH49">
+        <v>-0.110803324099727</v>
       </c>
     </row>
     <row r="50">
@@ -52264,6 +52565,9 @@
       <c r="FG50">
         <v>0.391236306729276</v>
       </c>
+      <c r="FH50">
+        <v>-2.80210157618214</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -52755,7 +53059,10 @@
         <v>-3.85852090032154</v>
       </c>
       <c r="FG51">
-        <v>0.0000000000000120024110770287</v>
+        <v>-1.35135135135135</v>
+      </c>
+      <c r="FH51">
+        <v>6.25</v>
       </c>
     </row>
     <row r="52">
@@ -53248,7 +53555,10 @@
         <v>2.86824021511801</v>
       </c>
       <c r="FG52">
-        <v>2.56410256410256</v>
+        <v>2.86935286935286</v>
+      </c>
+      <c r="FH52">
+        <v>1.66723375297721</v>
       </c>
     </row>
     <row r="53">
@@ -53741,7 +54051,10 @@
         <v>-0.957995578481933</v>
       </c>
       <c r="FG53">
-        <v>-1.53558052434458</v>
+        <v>-3.40823970037454</v>
+      </c>
+      <c r="FH53">
+        <v>-2.99057763211798</v>
       </c>
     </row>
     <row r="54">
@@ -54234,7 +54547,10 @@
         <v>-0.94786729857819</v>
       </c>
       <c r="FG54">
-        <v>-0.350262697022772</v>
+        <v>2.62697022767074</v>
+      </c>
+      <c r="FH54">
+        <v>3.44827586206896</v>
       </c>
     </row>
     <row r="55">
@@ -54727,7 +55043,10 @@
         <v>1.01941747572815</v>
       </c>
       <c r="FG55">
-        <v>-1.68509741969457</v>
+        <v>-2.63296471827276</v>
+      </c>
+      <c r="FH55">
+        <v>-1.1008111239861</v>
       </c>
     </row>
     <row r="56">
@@ -55220,7 +55539,10 @@
         <v>0.641025641025639</v>
       </c>
       <c r="FG56">
-        <v>0.347222222222215</v>
+        <v>-3.12500000000001</v>
+      </c>
+      <c r="FH56">
+        <v>-3.92156862745098</v>
       </c>
     </row>
   </sheetData>

</xml_diff>